<commit_message>
Refactor top news analysis to enhance relevance and clarity; update article titles, descriptions, and significance for improved user engagement.
</commit_message>
<xml_diff>
--- a/news_today.xlsx
+++ b/news_today.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1681" uniqueCount="1186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1685" uniqueCount="1189">
   <si>
     <t>Title</t>
   </si>
@@ -154,13 +154,13 @@
     <t>https://www.bbc.com/news/articles/c4g2d4l1x15o?at_medium=RSS&amp;at_campaign=rss</t>
   </si>
   <si>
-    <t>'I would sell a lung for a Hannah Montana tour': Fans react to 20th anniversary special announcement</t>
-  </si>
-  <si>
-    <t>Fans are gearing up for the "Hannahversary" - a special to mark the show's 20th anniversary.</t>
-  </si>
-  <si>
-    <t>https://www.bbc.com/news/articles/c0k1xjm7463o?at_medium=RSS&amp;at_campaign=rss</t>
+    <t>You're never too old, says dancer, 71, cast in Taylor Swift video</t>
+  </si>
+  <si>
+    <t>Denise Sides  was selected from hundreds of applicants to take part in the Opalite video.</t>
+  </si>
+  <si>
+    <t>https://www.bbc.com/news/articles/cly23mrv68ro?at_medium=RSS&amp;at_campaign=rss</t>
   </si>
   <si>
     <t>'Just push us into the sea': The frustration of a coastal community failed by political promises</t>
@@ -699,11 +699,11 @@
     <t>http://www.techmeme.com/260218/p32#a260218p32</t>
   </si>
   <si>
-    <t>Google unveils the $499 Pixel 10A, with a Tensor G4 and 8GB of RAM, like the Pixel 9A, an 11% brighter screen, and 128GB or 256GB storage, shipping from March 4 (Todd Haselton/The Verge)</t>
+    <t>Google unveils the $499 Pixel 10a, with a Tensor G4 and 8GB of RAM, like the Pixel 9a, an 11% brighter screen, and 128GB or 256GB storage, shipping from March 4 (Todd Haselton/The Verge)</t>
   </si>
   <si>
     <t xml:space="preserve">Todd Haselton / The Verge:
-Google unveils the $499 Pixel 10A, with a Tensor G4 and 8GB of RAM, like the Pixel 9A, an 11% brighter screen, and 128GB or 256GB storage, shipping from March 4  —  Google's midrange Pixels have been our top pick for budget Android phones for a while.  They offer good cameras and most of what you need at a budget-friendly price.</t>
+Google unveils the $499 Pixel 10a, with a Tensor G4 and 8GB of RAM, like the Pixel 9a, an 11% brighter screen, and 128GB or 256GB storage, shipping from March 4  —  Google's midrange Pixels have been our top pick for budget Android phones for a while.  They offer good cameras and most of what you need at a budget-friendly price.</t>
   </si>
   <si>
     <t>http://www.techmeme.com/260218/p31#a260218p31</t>
@@ -1700,6 +1700,267 @@
     <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQM3ZROU82Ykp2amNmUUR4LUxHUE9lMGc3Yk5qSG80aDFaeFgwZGVodWN4SWtXc295am42aHlyMTVmSjNRWmEtd1FrOHFmYmtkV3pfUE1fNkNhbktlTllfOHY4RnM5Q1pMV2l0Z0NhU1lJbFFtNWkwN181a0x2M281VWpvZmMtX3lzR0x3aUcydTBDUS1DcWRjSXpMbHh2XzVPT2JLWFVHUENjUFJrcU80?oc=5</t>
   </si>
   <si>
+    <t>Avalara Recognized on G2's 2026 Best Software Awards for Accounting and Finance Products - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Avalara Recognized on G2's 2026 Best Software Awards for Accounting and Finance Products  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPUE0yR3I5bkMzZDVvZlJIVk1ZSTBPa2YtRWswcnBPMXJrRElHRHc4VUk5b3ZWclZUcWNhcTdyaWVYcHhIUXdMWGJEZUhETFRTQUYwSjBhS1lkLUY5TGg5Y3RNU3RZWUNpRVJDX3RTdFlXZEN0MDZvNl83MGdYR3E0TVE0U0k?oc=5</t>
+  </si>
+  <si>
+    <t>Bank of America hikes stake in sinking crypto stock by 1,668% - Yahoo Finance Singapore</t>
+  </si>
+  <si>
+    <t>Bank of America hikes stake in sinking crypto stock by 1,668%  Yahoo Finance Singapore</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQSXJ5UEpsTjZuY2Fsa2c5M29OeTAzSlhScDZ0QnNxT3Rsd2w4ZThSZUNIaVhDdDFQSl81UVk1MmhLQzA0VTdYM0cyUkdXUWlTRlE1RVRYREcxNkJTNWZPOURoM2R0c1BQNmtPVGVzZFZGbFpXNmNlcmYzSGFqUVhMZUcwbFJWSFVi?oc=5</t>
+  </si>
+  <si>
+    <t>Billionaires’ Low Taxes Are Becoming a Problem for the Economy - The Wall Street Journal</t>
+  </si>
+  <si>
+    <t>Billionaires’ Low Taxes Are Becoming a Problem for the Economy  The Wall Street Journal</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMipANBVV95cUxPWkpTWUtnZWZzX3ZMMXFXdUpBemRacTZHaWl1bzk1d3ViRlpna0xpZHVqWktmcHdjQ3BKcVAzZThDdjdTM2xzdWxrRmZqQ1ljd0xyUXJSUkdyMjZ1SzlXMzVWem9KaXlyWlNpdHlrRVFJeXpaRFB5VVJoQUIwc3p6VXgwYlpFMGpGUVBlOE53TjBmVTkxX0dlM3N1WUw1eUw0dExCU3piS1pDUlBtTHZ3bHVmVkhZNXVYTjBpSm03TnRfYzVBLXR4dlp5YXNONmlQTldnWjVIbjlaMXpaa3RqRjl2WS1SQmVZRzFfWW5ucjdxUElYUVZXVE1rZmdvakRkVlZEcUlOSjY0TFlXSXR3TE9qS0J1cjZWS1hhM0hoMFBJLWhvNGF3NDhoZ2pDU1ZJVG4zNXl3clJabjljNGc1VWZBSVhqaGw5N1F2NmNEczlfbDM2UTBrVzM0ckIzV0ExT05UMXE0UkJIMHI3UkFPSW5sRDBaaF8yNGlVNHV1c1BPVEkxTDdsNjFUSTFVaXIxTjd4c1dSRUJZTjdaZnBKdG1nRi0?oc=5</t>
+  </si>
+  <si>
+    <t>Apollo-Backed Fund Lends Wayflyer $250 Million to Finance SMEs - Bloomberg.com</t>
+  </si>
+  <si>
+    <t>Apollo-Backed Fund Lends Wayflyer $250 Million to Finance SMEs  Bloomberg.com</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQ0FVYnZGaXlNek51bTVtd25PaWJqOFZZWmJqVF9qNUtTRjJIUEhRWTJtNG81YjVUUmZJMHpzWjJUXy1KQWJXUTBUelNxNV9tZGd5ZUtHa21CT2dGWGwzZTNwRWl4em5COWpNdjh4ZXpCWnVTNXpoME04S2R3cjdkSFluSTMzSmxJQ09VZWRsQjFvdXNnRUM0QTdCMTAzNG41YVR1Y2pjd0s5S1FCdHlXUllB?oc=5</t>
+  </si>
+  <si>
+    <t>Economic Sector Performance Dashboards - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Economic Sector Performance Dashboards  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiSkFVX3lxTE1aZHRnWXJQdlUwdmU4ZExFUzhEVXA5TXBHSFBsNS15TzJCSWtfMGRtU09HNENQMl9mTzlBenQyVmtTOFBKaFJDQ2ZB?oc=5</t>
+  </si>
+  <si>
+    <t>Coffee &amp; Donuts with the Mayor and Finance February 28 - City of West Chicago, Illinois</t>
+  </si>
+  <si>
+    <t>Coffee &amp; Donuts with the Mayor and Finance February 28  City of West Chicago, Illinois</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNR2VZNUNzbDNRYWNJMEVURm53elA3TU85SVdudUIzQ0Z5OTROdG44dXB5WlpqbkdPNHNSb044eHFvODZzQXJFTGJpM3NaajkyTTNid3ZVNjg0WldTaHA2eW5vRkdaWVBRUEttQnNqaGE4STFEZF9LQVhlRHdmTlc3ZVRscXRkMExyREE?oc=5</t>
+  </si>
+  <si>
+    <t>Governor Moore Testifies Before Senate Finance Committee in Support of Legislative Agenda to Make Maryland More Affordable and More Competitive - Office of Governor Wes Moore (.gov)</t>
+  </si>
+  <si>
+    <t>Governor Moore Testifies Before Senate Finance Committee in Support of Legislative Agenda to Make Maryland More Affordable and More Competitive  Office of Governor Wes Moore (.gov)</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMihgJBVV95cUxQM1pHd3I0RG5XejdpVWJEcUxramNPeU1WOUxlU0MyczlaS0pLMUw2Tm1nSVQzcGNPRWpQT1I3cXVLcXBUaUpYcGxGSkg3OHp1U3Y2eDZhV2RtRV9FR3J6QUV6Y2hyblRGeVNkdU1HT0ZEOFc4Q1RhREJCN29JVlptRzk2TWZoaHhncjhwekdHb0xTVTFMMjBDUnl2QmtqOXBpUmgyaUlTaE1XeW5WOVJDaWR0X3NPaXZieDd3MjREM3NCYU0wSzBWVGptbDhUWGIwcVFDUHdvTmhRdnBQd21HazlmTDRBUGx3VDdrZE02b01PZG1JeFpLMlJPTTd3Y21DSFNIZ2Zn?oc=5</t>
+  </si>
+  <si>
+    <t>Avalara Recognized on G2's 2026 Best Software Awards for Accounting and Finance Products - PR Newswire</t>
+  </si>
+  <si>
+    <t>Avalara Recognized on G2's 2026 Best Software Awards for Accounting and Finance Products  PR Newswire</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOOExlVW1PTkhpeVRVeVJqS1A3WVdydlhPNGx5cWhmZS1TQ3pBM3hnZGZwSFhkVWtnRnlRNm1tcnlySzVnYk5uZVRrbVNSV3BMQXEwTkhJTTZweVlZVWpxcndnZ0pxcGdhOTBJQ25MY1lKcm9WdnZWaldvMVR6cnhCNEl1aVBaVDRrTGgwMmVHMl9jQVIwc3pZeHVVTGVDb2hpZTAwa3M0MFcwRWhuaW81R0JIY2JEanRpc0c0aFB2dGs0OTZQSDhIVUhHSjByeWFuMEZ0eHBEbzVIX1k?oc=5</t>
+  </si>
+  <si>
+    <t>Program - Milken Institute</t>
+  </si>
+  <si>
+    <t>Program  Milken Institute</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE9rdkpHVDFFMmpRcTFFc0FlTnJ2bElINVdKNm1OeDVVWXVVMl8yVnpETHpKalVCc2o2T3NtSVhVWlBodzBVdFZycTQ5MksxbWFIbXh2eC1wbWNOMUt6MkxQcHdiTFdxZFBhQ2JQUFNKUQ?oc=5</t>
+  </si>
+  <si>
+    <t>Konica Minolta Wins the Bronze Prize in the Seventh ESG Finance Awards Japan of the Ministry of the Environment - Konica Minolta</t>
+  </si>
+  <si>
+    <t>Konica Minolta Wins the Bronze Prize in the Seventh ESG Finance Awards Japan of the Ministry of the Environment  Konica Minolta</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE1XVnlJT3NZTlNITVVJU2JrUV9yejAtMTIxa05DXzY4ME0zWVBoRTBvOUduLWp1OTR4N21EbkdOa1VCQjBqYURmUUpVQ0p6VzZSX1BfMENPRTBScFpFSGxsRGloZzlPY1pVak9qNWNiMmVfLWNVdzhXVQ?oc=5</t>
+  </si>
+  <si>
+    <t>Women in Securities Finance appoints Hill Sands - Securities Finance Times</t>
+  </si>
+  <si>
+    <t>Women in Securities Finance appoints Hill Sands  Securities Finance Times</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQMjJkLTZVcm84eTNLM3RfeFl2d21odEx4ZlJSNUtUSkpPVzVockVkRmtOY00xcGg4VFltTXNoUFJRVkVFX0habzNBMlZNN3RmODJLc0R6djdOOWkteGtPb3FfazcwbUQ2MDlUTjNTaEJuM0IycDdKSUJHak5LbFNxeEFDMGVRWXJYTTFsQlRoRWcwWlQ5X1FQUnVEend5R1B2ejUw?oc=5</t>
+  </si>
+  <si>
+    <t>The Real Bottleneck in Finance Isn’t Payments. It’s Settlement. - FinTech Weekly</t>
+  </si>
+  <si>
+    <t>The Real Bottleneck in Finance Isn’t Payments. It’s Settlement.  FinTech Weekly</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOR3RLRlRYOFVvWE9LX1c1UzRubldLcjg1eXpSbXE3YlNvb2U3ZVdQZWZFVnBYOHhWYkNSN0JKZ2t0MFdSRGVLUmRtYmFxbUEzM0hBNXFmYlJJbEZZNUMwbkpFazNVNUdTTklFVmg4N3NGX2JUWDFpRV9ScXRRWG9pa1A1Q1pxc093U2c?oc=5</t>
+  </si>
+  <si>
+    <t>New Climate Finance Initiative Supports Climate Adaptation Efforts in Glacier-Dependent Regions - Columbia University in the City of New York</t>
+  </si>
+  <si>
+    <t>New Climate Finance Initiative Supports Climate Adaptation Efforts in Glacier-Dependent Regions  Columbia University in the City of New York</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOMTN2TUpQT0dqaGR5VU9SSng0YzJibE1DZGdJOUVVWm4xM0RDVkUteVBpS0lZb3k5VDhxVEsyekNWNXUzR2YtN3pOV2hNRDQ4WVI5VHpyaDNnVXNmc21CNlh4SDdJd0V3V3dyWU9hc3VObGotYmZvQzNrWVRRTUFCSUVTU2Zial9JRWU0c1ZNZWw1eFFCdmxFZ2JxdDJkLWNxa0NEM2lFUlFtdkNHSjZQeWUwNl81TEJCdkY4QnVwb2JIRmE4ZGlGUVNaQ3FFN1BIb2k2RG5FbU8?oc=5</t>
+  </si>
+  <si>
+    <t>AI adoption already hitting Irish graduate jobs, finance department says - Reuters</t>
+  </si>
+  <si>
+    <t>AI adoption already hitting Irish graduate jobs, finance department says  Reuters</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNY0ZlYUU3ZWpFUFF0WEk1eXRkc1ZwbUduSUpVdjJoeXdLeWhJVnMzV0taTk11b0lpeklmMzZBM29YVmd6V3dqWlhENkJnZ0dRRjdNSWd3TVV5dURwbUM3QjFzem1wSHd2Y0Y2aU5GWFcyS2tSR3RsTmVfQ1ZzWWFvbU5Ld05YYlBiTVNmMm5rVGxHVEVDcjJzUVM4RjZxQ1gtbWp5clFFalNZbmtMWThuZzFDczlsSjA?oc=5</t>
+  </si>
+  <si>
+    <t>Symposium on International Investment Law &amp; Contemporary Crises: Energy Finance Market Design &amp; IIA Claims - Opinio Juris</t>
+  </si>
+  <si>
+    <t>Symposium on International Investment Law &amp; Contemporary Crises: Energy Finance Market Design &amp; IIA Claims  Opinio Juris</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNdE85WEhsdkw2YTBwVW14aklibzR3X0pLUVVkZEVlM2xjNEFzRXBzMkVINmQyc1VZMExFV0R1WmRCZHlac2FzQS03djdrSk9SdU1sM1ZOS2JlSGRGS0RDU3lQaktUNlBPN0VVclhWbjdJUXdkalVPM0stRXp4S3luVUJRNkVyV2NnUVpoTHhQM2VVV3F2QzBfT2VUNDNyVENwQWJyNV82TldkZE1ITnNiWGVhRGM1TlA1Z3NPcHJ4Rjg4S1pSeXFXNjc2Wlh6X21obUE?oc=5</t>
+  </si>
+  <si>
+    <t>How Credit Cards Keep America’s Small Businesses Running Strong - U.S. Chamber of Commerce</t>
+  </si>
+  <si>
+    <t>How Credit Cards Keep America’s Small Businesses Running Strong  U.S. Chamber of Commerce</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOOEZRTVRzZlF2RzVaVVZXdm55a1JWRzlHenl6OWQ4czBNa0hLbFF1dWdFMXI4RExnQVhmQWpzb2tEanNvNEU1UzQ5ZXRhaXgzY3BUazl3WFdkb1VwMGowMkl2eEhoT0x1djA1LVltOTZOWlBTOXQ5YzItUkRLcmhXd0RvRHhkZi0tZERvX19FWUpEazZwdHlhVDZZekk?oc=5</t>
+  </si>
+  <si>
+    <t>BBVA welcomes Shepherd - Securities Finance Times</t>
+  </si>
+  <si>
+    <t>BBVA welcomes Shepherd  Securities Finance Times</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxORVBDSXlvSTBQR0w4WTc1WkhzNDdGMmhuSWlpOE82Mm5uTnBNVnBUTUJSMWVuNUp4OXVGdV90M0pZelBNcXBUdmZOVWQtVlN2eWV4bFpBSG1ZcFN2eHNSS1hJam90R0dRWXRROEtsLXlRMTVWcFJtVGdSR3FpNWZkRjN4ekRlZUU4cEJvTmtUUVdwLS11T1RuN1F6UWJxcFJ5UXBZ?oc=5</t>
+  </si>
+  <si>
+    <t>Troutman Pepper Locke Weekly Consumer Financial Services Newsletter – February 18, 2026 - Consumer Financial Services Law Monitor</t>
+  </si>
+  <si>
+    <t>Troutman Pepper Locke Weekly Consumer Financial Services Newsletter – February 18, 2026  Consumer Financial Services Law Monitor</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPUExOOWVkYWxmODJERVdlUlpCOFhXdDFmTXVWdW54TnFhOWZvNUdBWERLVnd3aXR5aFNwaHk1QnVSZVREVzkybjhoemhPYTNhVkZQdFFlelJmS19vQV9ZNWxVVE9SN05mVEtaVDV0b1ZvNHRXazI0TmFLX1c1TFVkNnUxVExBbnFCVWZwLTA0NTJFS3BjRWk5TWRGa3JHRTFxa2JfSm11WC1OdEtEWHZ5Mzc0V1NXSC1mVW5HUUtjTlJ2bGpQOEIwUzlmcGF2dXNoMHFzTnVLeVM3RXBlOXc?oc=5</t>
+  </si>
+  <si>
+    <t>Earnings live: Palo Alto Networks stock sinks after company cuts full-year forecast - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Earnings live: Palo Alto Networks stock sinks after company cuts full-year forecast  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxQVWE1S2hNazUwaEp3UTQ4ZWcwY1FXY2JnVG4yQ2ZQeTRVdUxKdVhFcDBDZnFzTmNNRUFIMWJPek80ZTNKS2VqWFAzTEVPXzREN1kzQnVzZkdvMG5qN1VOR2dVNFBnSzdEaGVUUmI5TGhBbGFwQUJIVno5bHc0YzdBck9SNjRBcnNwRndFTFN0dGFId01wVlU4bEhGOUNSRUN6aEIwNnByeGJnd3FiM2ZXMkQ4X0FnZ0xQeHJlRWd2UFphNFBIeDBDNlpVeWNOQQ?oc=5</t>
+  </si>
+  <si>
+    <t>Nvidia and Meta expand GPU team up with millions of additional AI chips - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Nvidia and Meta expand GPU team up with millions of additional AI chips  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNaEc1R3NCLTZRdDgwVWd6UDR5ZXB5SXd4Q0c2dlBUbVpnT1ZzRU8xMnh5bWNEa1BuS25zRHg3Qk45OW1QaVk3MlE1MEhta25icVhvYkw5UXd0MjU2U2gtVmljdFBrMzM1X1FKQzRPNG9uVllMb0lRSXFvQWx3TWFmaDAyaTNIMFhabl9maFdRek1jcVpBOEJaeFMzbUgxbF82dXRKTjVCZzRqZm9iNkUwbjNyQmZ6WkYw?oc=5</t>
+  </si>
+  <si>
+    <t>Chicago Atlantic Real Estate Finance Schedules Fourth Quarter 2025 Earnings Release and Conference Call Date - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Chicago Atlantic Real Estate Finance Schedules Fourth Quarter 2025 Earnings Release and Conference Call Date  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNazBfQm5fMm1UTGZMVF9JQm5FLXNnZHpwekp6R3lNQTk5aGYtd2J2eW9KemNpSHZWNzQtVVZ6NU92dTh6eEFSOTZ5NThjeV9yd0VXMU43djVCQTBLYUhJeks1b2xXX21HYXdVNjFOdzNwZDRrNmlRX1dFTGNyUjYtMHZPUUVaTWo5bWc?oc=5</t>
+  </si>
+  <si>
+    <t>Stock market today: Dow, S&amp;P 500, Nasdaq rise as AI worries recede, with Fed minutes ahead - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Stock market today: Dow, S&amp;P 500, Nasdaq rise as AI worries recede, with Fed minutes ahead  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQcEhkYkxjdlVSbDVfTk83VmVuZ2pVTmgzNjFsRFRjc0VqelNPX1c1RFZ4am1Ra3U5TUlVWnFNTVZkTlNTRGpzanNCcUVybTlGNHNMaXR4ajc4VVZqbW55cFp5ZWJlR3NGZmM1OFEyMmFqblBQVmNwdkdLRzRSMWdfVVpwZmYyRndHczgtOHYxWTNSQ3V1WmkzcTJod0d6X0pmY3B2d0ItTmx1OWpCenVtdzUtc09PeW1JWVgwcDQxYUJIZktZRHBGTC1idnc2cFFINVE?oc=5</t>
+  </si>
+  <si>
+    <t>Snap Finance Study Finds Majority of U.S. Households Delayed Essential Purchases in 2025 as Credit Pressures Persist Into 2026 - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Snap Finance Study Finds Majority of U.S. Households Delayed Essential Purchases in 2025 as Credit Pressures Persist Into 2026  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxOTzNzdHpaNkF0TUlxNHJwdGtIRzQzdTBlNXpkUWRTbVdna1M0eE1IU1NvS1otYTAzVEFub2lvVWlKeHd6QkY3RmJ0T3NqSkVBX29Ya25DbkNydnZDRG55OGxDTksydXo4Y3JWSXNRd1U3UUY5Zm0zdlExbDVkZkxzVmxlU05Rdw?oc=5</t>
+  </si>
+  <si>
+    <t>Are Finance Stocks Lagging Barclays (BCS) This Year? - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Are Finance Stocks Lagging Barclays (BCS) This Year?  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPbkt4OTRYNGtDSjRKUTF5Y3hVZ242YzN0Nmlub0kzMl9KbnRRU00tMHdLVEl3aTY0V0Y5QWFzRDAtQ0M5WlVGV3ZxV1NzN3VpaWt2UVhVNWZVTDlScHA1bzg5TFlpN2p4Q0FGbHVhVVNuaWNzOTVQMTVoeklfR1hOT3h0R1ZlYmpQ?oc=5</t>
+  </si>
+  <si>
+    <t>Unlocking Finance for Nature-based Solutions in Indian Cities - Climate Policy Initiative</t>
+  </si>
+  <si>
+    <t>Unlocking Finance for Nature-based Solutions in Indian Cities  Climate Policy Initiative</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNbE9VZDZKVktsajJEVG0yM1ZfWEJ3Ums3RHRTM0FOZTFEZnFwa1NFSXBSbXpLMUpzNUktWGtqSzRVN052RllQUDNMY2x3TWlFSnNUS2VyNzF5X05ZWmx1MTlYSVlwOS05WDhjcmpCZTBacHc1Q29Ba2lZUkVuclMtaFJ6ejI3Z2lkMHVYdEFJREJIdXF2ZUVXT0VMMlFaLWRoeHFKY2xMS2syRTJWZDVQaVRraTQ?oc=5</t>
+  </si>
+  <si>
+    <t>West Virginia Senate Finance Committee approves appropriations bill for Hancock County Schools - News and Sentinel</t>
+  </si>
+  <si>
+    <t>West Virginia Senate Finance Committee approves appropriations bill for Hancock County Schools  News and Sentinel</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxORmNQWEtJSnc0OEQ2Yl92TldtMHJrVEdaZUdNdHNvb0pWdmpLcGdTV0xXZE5EcmJsWWFLSmxaOENUdUFqel92bTRjZ1g0TU9uLXVHTXNTY2x0VmVYV1Y4V1p4RTZKVDVNUGZHY0l3V3dWdmtuVGxMcmtOQVpralpLaDdGNXJ6OUt6dEpsMlNHQzNSOXpsclJBX1lOMXYzdkptaGlJRkRhNVdIaWowc2pFTTM5VlRFVlJsM0FCaU81TDl0by1fVVRCcUhYdThWYUdJbVRwUElna0hEVjQtM0NhYUlBcUtBUQ?oc=5</t>
+  </si>
+  <si>
+    <t>Lightrock grabs an exit opportunity from Indian small business lender Aye Finance - ImpactAlpha</t>
+  </si>
+  <si>
+    <t>Lightrock grabs an exit opportunity from Indian small business lender Aye Finance  ImpactAlpha</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPbW5lcmJoSERuOFp0MGYzaHJXS2Q4c2FTNUgyODYybUlOZ2JKUlVLcTcwYlRoNmRxbC0tejNBZXFaSHhEaTR2Q1VDT1BEREtLWjhiM2JDSFFpM2JGMUYyazI4a2ZkTm9Ja2pCRmNtcGhqTlJzcFowVlNKWmxtOHpSR1g1X1hEaXZyVXB1Y0ZlYVlkV3N3VTVTT2U3Y1ZKMHE2VkNSeHpKNWYtUQ?oc=5</t>
+  </si>
+  <si>
+    <t>OPENLANE, Inc. Reports 2025 Financial Results - PR Newswire</t>
+  </si>
+  <si>
+    <t>OPENLANE, Inc. Reports 2025 Financial Results  PR Newswire</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNZ3FFQzNzUG81QkNjTDgycHBKSUh3NURtVi1WUkR0cGFoODg3LUFyX25YYjVYNFIzU0U2cW9YT2pkcUNxTnpWb2VoUFpGTGI2N2I0Y2tmZ1hwWVlQRzhNVU1LdnBzYkx6QUpKSlRLQmJiMHFuV0NSNkhpTEZpVTIxeTRwVmUxc2c3S01fYnVWZVJDR2Z3VzlvV2MweUw0bXJk?oc=5</t>
+  </si>
+  <si>
+    <t>Financial scams are on the rise — but what’s being done about it? - The Hill</t>
+  </si>
+  <si>
+    <t>Financial scams are on the rise — but what’s being done about it?  The Hill</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQbFU0OFZxQ2tVdlpqamVrdldYbTE1N0NkOWw4RjlnQ3lDaFVIanpfTFNrbllSVWMySl9DS0FmZzlWSDRCTEloTEF2Vms5QmRPaFpJcjM0T3RTa3JtY3UtbW1tVlpHQkxYYWRlTTI4NWMwaXp2SVdYZDdZUlRYMHV4RmVXWdIBiAFBVV95cUxOZ1ZOWTllSWJKWEFaLTl4ZEk4LUx5dzl3M2tiMEhKZWhLb0dpaW16QnJ3RzRudExGS2NPeGZjYVVBbnItVGxfNE1pWUxyZG1SMmMxSEdxSVhIZndmM0FpRDdTbFFrNHluWVh6a2M5T3RRT2FsdkdJdlhJaGc1WXp1dVNFNXhlQ2hI?oc=5</t>
+  </si>
+  <si>
     <t>Is Synchrony Financial (SYF) Still Attractive After Recent Share Price Pullback? - Yahoo Finance</t>
   </si>
   <si>
@@ -1709,247 +1970,67 @@
     <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQYzJRV0I4UzFRZ2ljeTFwanMwOGZVZ1lIZ05KbUh4QUJCVEM5SDVtMUhmQXl0VDAybUZvMHJTbTVCTEZPTVBnZE5xb2ZWWnRKWXBram52aDZiMGJxeTlfb0l1SldpU2t2RUlCZEpLOEdORUxlQ3FMZWNzbS1oOE5FbUxLUWRMaV8tQkdZTUNfcw?oc=5</t>
   </si>
   <si>
-    <t>Avalara Recognized on G2's 2026 Best Software Awards for Accounting and Finance Products - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Avalara Recognized on G2's 2026 Best Software Awards for Accounting and Finance Products  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPUE0yR3I5bkMzZDVvZlJIVk1ZSTBPa2YtRWswcnBPMXJrRElHRHc4VUk5b3ZWclZUcWNhcTdyaWVYcHhIUXdMWGJEZUhETFRTQUYwSjBhS1lkLUY5TGg5Y3RNU3RZWUNpRVJDX3RTdFlXZEN0MDZvNl83MGdYR3E0TVE0U0k?oc=5</t>
-  </si>
-  <si>
-    <t>Billionaires’ Low Taxes Are Becoming a Problem for the Economy - The Wall Street Journal</t>
-  </si>
-  <si>
-    <t>Billionaires’ Low Taxes Are Becoming a Problem for the Economy  The Wall Street Journal</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMipANBVV95cUxNNjVTREItcVAtQk9uZksyTWQyUUx5a1Vwc2VWRllHM2FzODNVWGQ1RkQ5NnRaRTAtTzRFd1c0U01ReksyRmRrLXFHRUl3V3VlWHdTY0RJVW94Y1RPT25RSVFrSFdaWE5NZU9kMkhVMU44Sm1EMU5KTGNXTm1ZaDJzZldFV3hkakJSVzlaVm1UeldLOWtsZFRxNzBVV0hYOFFNVWZ6aE9uNzN1V0FiTlRLNk95OWFaVEdmekF3WUtCaHZJNmx6bFoxczJiVF9qVzJYZVZYSlh2dDdtWTJYQnR1ZTlwazU0ZVJTYjZZQTBZRFNjcDU1R09LR0stWHVVQnN4dENaMTMyY3ZPS2xSTWFZUkFSNDZiWHZGM25QVXBwaXE3SkhEM09xQ0QyZ2VqaXVoQUNydHNiNEFjQ1M3NmY5b2hCVnZWX1dYUmxhY3I2THhyekxXa1d4NnBIYlVYRXo1OElzd1hCamhXdkJTcklnemdSNm5pSi1FSVNJaS1rbHRqa3RvM0ZMTThNV01RLUdkWUNPVndOQ3JJdHNqakNDdmNKa1Y?oc=5</t>
-  </si>
-  <si>
-    <t>Apollo-Backed Fund Lends Wayflyer $250 Million to Finance SMEs - Bloomberg.com</t>
-  </si>
-  <si>
-    <t>Apollo-Backed Fund Lends Wayflyer $250 Million to Finance SMEs  Bloomberg.com</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPQ0FVYnZGaXlNek51bTVtd25PaWJqOFZZWmJqVF9qNUtTRjJIUEhRWTJtNG81YjVUUmZJMHpzWjJUXy1KQWJXUTBUelNxNV9tZGd5ZUtHa21CT2dGWGwzZTNwRWl4em5COWpNdjh4ZXpCWnVTNXpoME04S2R3cjdkSFluSTMzSmxJQ09VZWRsQjFvdXNnRUM0QTdCMTAzNG41YVR1Y2pjd0s5S1FCdHlXUllB?oc=5</t>
-  </si>
-  <si>
-    <t>Economic Sector Performance Dashboards - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Economic Sector Performance Dashboards  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiSkFVX3lxTE1aZHRnWXJQdlUwdmU4ZExFUzhEVXA5TXBHSFBsNS15TzJCSWtfMGRtU09HNENQMl9mTzlBenQyVmtTOFBKaFJDQ2ZB?oc=5</t>
-  </si>
-  <si>
-    <t>Coffee &amp; Donuts with the Mayor and Finance February 28 - City of West Chicago, Illinois</t>
-  </si>
-  <si>
-    <t>Coffee &amp; Donuts with the Mayor and Finance February 28  City of West Chicago, Illinois</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNR2VZNUNzbDNRYWNJMEVURm53elA3TU85SVdudUIzQ0Z5OTROdG44dXB5WlpqbkdPNHNSb044eHFvODZzQXJFTGJpM3NaajkyTTNid3ZVNjg0WldTaHA2eW5vRkdaWVBRUEttQnNqaGE4STFEZF9LQVhlRHdmTlc3ZVRscXRkMExyREE?oc=5</t>
-  </si>
-  <si>
-    <t>Governor Moore Testifies Before Senate Finance Committee in Support of Legislative Agenda to Make Maryland More Affordable and More Competitive - Office of Governor Wes Moore (.gov)</t>
-  </si>
-  <si>
-    <t>Governor Moore Testifies Before Senate Finance Committee in Support of Legislative Agenda to Make Maryland More Affordable and More Competitive  Office of Governor Wes Moore (.gov)</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMihgJBVV95cUxQM1pHd3I0RG5XejdpVWJEcUxramNPeU1WOUxlU0MyczlaS0pLMUw2Tm1nSVQzcGNPRWpQT1I3cXVLcXBUaUpYcGxGSkg3OHp1U3Y2eDZhV2RtRV9FR3J6QUV6Y2hyblRGeVNkdU1HT0ZEOFc4Q1RhREJCN29JVlptRzk2TWZoaHhncjhwekdHb0xTVTFMMjBDUnl2QmtqOXBpUmgyaUlTaE1XeW5WOVJDaWR0X3NPaXZieDd3MjREM3NCYU0wSzBWVGptbDhUWGIwcVFDUHdvTmhRdnBQd21HazlmTDRBUGx3VDdrZE02b01PZG1JeFpLMlJPTTd3Y21DSFNIZ2Zn?oc=5</t>
-  </si>
-  <si>
-    <t>Avalara Recognized on G2's 2026 Best Software Awards for Accounting and Finance Products - PR Newswire</t>
-  </si>
-  <si>
-    <t>Avalara Recognized on G2's 2026 Best Software Awards for Accounting and Finance Products  PR Newswire</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOOExlVW1PTkhpeVRVeVJqS1A3WVdydlhPNGx5cWhmZS1TQ3pBM3hnZGZwSFhkVWtnRnlRNm1tcnlySzVnYk5uZVRrbVNSV3BMQXEwTkhJTTZweVlZVWpxcndnZ0pxcGdhOTBJQ25MY1lKcm9WdnZWaldvMVR6cnhCNEl1aVBaVDRrTGgwMmVHMl9jQVIwc3pZeHVVTGVDb2hpZTAwa3M0MFcwRWhuaW81R0JIY2JEanRpc0c0aFB2dGs0OTZQSDhIVUhHSjByeWFuMEZ0eHBEbzVIX1k?oc=5</t>
-  </si>
-  <si>
-    <t>Program - Milken Institute</t>
-  </si>
-  <si>
-    <t>Program  Milken Institute</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE9rdkpHVDFFMmpRcTFFc0FlTnJ2bElINVdKNm1OeDVVWXVVMl8yVnpETHpKalVCc2o2T3NtSVhVWlBodzBVdFZycTQ5MksxbWFIbXh2eC1wbWNOMUt6MkxQcHdiTFdxZFBhQ2JQUFNKUQ?oc=5</t>
-  </si>
-  <si>
-    <t>Konica Minolta Wins the Bronze Prize in the Seventh ESG Finance Awards Japan of the Ministry of the Environment - Konica Minolta</t>
-  </si>
-  <si>
-    <t>Konica Minolta Wins the Bronze Prize in the Seventh ESG Finance Awards Japan of the Ministry of the Environment  Konica Minolta</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE1XVnlJT3NZTlNITVVJU2JrUV9yejAtMTIxa05DXzY4ME0zWVBoRTBvOUduLWp1OTR4N21EbkdOa1VCQjBqYURmUUpVQ0p6VzZSX1BfMENPRTBScFpFSGxsRGloZzlPY1pVak9qNWNiMmVfLWNVdzhXVQ?oc=5</t>
-  </si>
-  <si>
-    <t>New Climate Finance Initiative Supports Climate Adaptation Efforts in Glacier-Dependent Regions - Columbia University in the City of New York</t>
-  </si>
-  <si>
-    <t>New Climate Finance Initiative Supports Climate Adaptation Efforts in Glacier-Dependent Regions  Columbia University in the City of New York</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOMTN2TUpQT0dqaGR5VU9SSng0YzJibE1DZGdJOUVVWm4xM0RDVkUteVBpS0lZb3k5VDhxVEsyekNWNXUzR2YtN3pOV2hNRDQ4WVI5VHpyaDNnVXNmc21CNlh4SDdJd0V3V3dyWU9hc3VObGotYmZvQzNrWVRRTUFCSUVTU2Zial9JRWU0c1ZNZWw1eFFCdmxFZ2JxdDJkLWNxa0NEM2lFUlFtdkNHSjZQeWUwNl81TEJCdkY4QnVwb2JIRmE4ZGlGUVNaQ3FFN1BIb2k2RG5FbU8?oc=5</t>
-  </si>
-  <si>
-    <t>Women in Securities Finance appoints Hill Sands - Securities Finance Times</t>
-  </si>
-  <si>
-    <t>Women in Securities Finance appoints Hill Sands  Securities Finance Times</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQMjJkLTZVcm84eTNLM3RfeFl2d21odEx4ZlJSNUtUSkpPVzVockVkRmtOY00xcGg4VFltTXNoUFJRVkVFX0habzNBMlZNN3RmODJLc0R6djdOOWkteGtPb3FfazcwbUQ2MDlUTjNTaEJuM0IycDdKSUJHak5LbFNxeEFDMGVRWXJYTTFsQlRoRWcwWlQ5X1FQUnVEend5R1B2ejUw?oc=5</t>
-  </si>
-  <si>
-    <t>The Real Bottleneck in Finance Isn’t Payments. It’s Settlement. - FinTech Weekly</t>
-  </si>
-  <si>
-    <t>The Real Bottleneck in Finance Isn’t Payments. It’s Settlement.  FinTech Weekly</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOR3RLRlRYOFVvWE9LX1c1UzRubldLcjg1eXpSbXE3YlNvb2U3ZVdQZWZFVnBYOHhWYkNSN0JKZ2t0MFdSRGVLUmRtYmFxbUEzM0hBNXFmYlJJbEZZNUMwbkpFazNVNUdTTklFVmg4N3NGX2JUWDFpRV9ScXRRWG9pa1A1Q1pxc093U2c?oc=5</t>
-  </si>
-  <si>
-    <t>Symposium on International Investment Law &amp; Contemporary Crises: Energy Finance Market Design &amp; IIA Claims - Opinio Juris</t>
-  </si>
-  <si>
-    <t>Symposium on International Investment Law &amp; Contemporary Crises: Energy Finance Market Design &amp; IIA Claims  Opinio Juris</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNdE85WEhsdkw2YTBwVW14aklibzR3X0pLUVVkZEVlM2xjNEFzRXBzMkVINmQyc1VZMExFV0R1WmRCZHlac2FzQS03djdrSk9SdU1sM1ZOS2JlSGRGS0RDU3lQaktUNlBPN0VVclhWbjdJUXdkalVPM0stRXp4S3luVUJRNkVyV2NnUVpoTHhQM2VVV3F2QzBfT2VUNDNyVENwQWJyNV82TldkZE1ITnNiWGVhRGM1TlA1Z3NPcHJ4Rjg4S1pSeXFXNjc2Wlh6X21obUE?oc=5</t>
-  </si>
-  <si>
-    <t>AI adoption already hitting Irish graduate jobs, finance department says - Reuters</t>
-  </si>
-  <si>
-    <t>AI adoption already hitting Irish graduate jobs, finance department says  Reuters</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNY0ZlYUU3ZWpFUFF0WEk1eXRkc1ZwbUduSUpVdjJoeXdLeWhJVnMzV0taTk11b0lpeklmMzZBM29YVmd6V3dqWlhENkJnZ0dRRjdNSWd3TVV5dURwbUM3QjFzem1wSHd2Y0Y2aU5GWFcyS2tSR3RsTmVfQ1ZzWWFvbU5Ld05YYlBiTVNmMm5rVGxHVEVDcjJzUVM4RjZxQ1gtbWp5clFFalNZbmtMWThuZzFDczlsSjA?oc=5</t>
-  </si>
-  <si>
-    <t>How Credit Cards Keep America’s Small Businesses Running Strong - U.S. Chamber of Commerce</t>
-  </si>
-  <si>
-    <t>How Credit Cards Keep America’s Small Businesses Running Strong  U.S. Chamber of Commerce</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOOEZRTVRzZlF2RzVaVVZXdm55a1JWRzlHenl6OWQ4czBNa0hLbFF1dWdFMXI4RExnQVhmQWpzb2tEanNvNEU1UzQ5ZXRhaXgzY3BUazl3WFdkb1VwMGowMkl2eEhoT0x1djA1LVltOTZOWlBTOXQ5YzItUkRLcmhXd0RvRHhkZi0tZERvX19FWUpEazZwdHlhVDZZekk?oc=5</t>
-  </si>
-  <si>
-    <t>Troutman Pepper Locke Weekly Consumer Financial Services Newsletter – February 18, 2026 - Consumer Financial Services Law Monitor</t>
-  </si>
-  <si>
-    <t>Troutman Pepper Locke Weekly Consumer Financial Services Newsletter – February 18, 2026  Consumer Financial Services Law Monitor</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPUExOOWVkYWxmODJERVdlUlpCOFhXdDFmTXVWdW54TnFhOWZvNUdBWERLVnd3aXR5aFNwaHk1QnVSZVREVzkybjhoemhPYTNhVkZQdFFlelJmS19vQV9ZNWxVVE9SN05mVEtaVDV0b1ZvNHRXazI0TmFLX1c1TFVkNnUxVExBbnFCVWZwLTA0NTJFS3BjRWk5TWRGa3JHRTFxa2JfSm11WC1OdEtEWHZ5Mzc0V1NXSC1mVW5HUUtjTlJ2bGpQOEIwUzlmcGF2dXNoMHFzTnVLeVM3RXBlOXc?oc=5</t>
-  </si>
-  <si>
-    <t>BBVA welcomes Shepherd - Securities Finance Times</t>
-  </si>
-  <si>
-    <t>BBVA welcomes Shepherd  Securities Finance Times</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxORVBDSXlvSTBQR0w4WTc1WkhzNDdGMmhuSWlpOE82Mm5uTnBNVnBUTUJSMWVuNUp4OXVGdV90M0pZelBNcXBUdmZOVWQtVlN2eWV4bFpBSG1ZcFN2eHNSS1hJam90R0dRWXRROEtsLXlRMTVWcFJtVGdSR3FpNWZkRjN4ekRlZUU4cEJvTmtUUVdwLS11T1RuN1F6UWJxcFJ5UXBZ?oc=5</t>
-  </si>
-  <si>
-    <t>Earnings live: Palo Alto Networks stock sinks after company cuts full-year forecast - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Earnings live: Palo Alto Networks stock sinks after company cuts full-year forecast  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxQVWE1S2hNazUwaEp3UTQ4ZWcwY1FXY2JnVG4yQ2ZQeTRVdUxKdVhFcDBDZnFzTmNNRUFIMWJPek80ZTNKS2VqWFAzTEVPXzREN1kzQnVzZkdvMG5qN1VOR2dVNFBnSzdEaGVUUmI5TGhBbGFwQUJIVno5bHc0YzdBck9SNjRBcnNwRndFTFN0dGFId01wVlU4bEhGOUNSRUN6aEIwNnByeGJnd3FiM2ZXMkQ4X0FnZ0xQeHJlRWd2UFphNFBIeDBDNlpVeWNOQQ?oc=5</t>
-  </si>
-  <si>
-    <t>Nvidia and Meta expand GPU team up with millions of additional AI chips - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Nvidia and Meta expand GPU team up with millions of additional AI chips  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNaEc1R3NCLTZRdDgwVWd6UDR5ZXB5SXd4Q0c2dlBUbVpnT1ZzRU8xMnh5bWNEa1BuS25zRHg3Qk45OW1QaVk3MlE1MEhta25icVhvYkw5UXd0MjU2U2gtVmljdFBrMzM1X1FKQzRPNG9uVllMb0lRSXFvQWx3TWFmaDAyaTNIMFhabl9maFdRek1jcVpBOEJaeFMzbUgxbF82dXRKTjVCZzRqZm9iNkUwbjNyQmZ6WkYw?oc=5</t>
-  </si>
-  <si>
-    <t>Chicago Atlantic Real Estate Finance Schedules Fourth Quarter 2025 Earnings Release and Conference Call Date - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Chicago Atlantic Real Estate Finance Schedules Fourth Quarter 2025 Earnings Release and Conference Call Date  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNazBfQm5fMm1UTGZMVF9JQm5FLXNnZHpwekp6R3lNQTk5aGYtd2J2eW9KemNpSHZWNzQtVVZ6NU92dTh6eEFSOTZ5NThjeV9yd0VXMU43djVCQTBLYUhJeks1b2xXX21HYXdVNjFOdzNwZDRrNmlRX1dFTGNyUjYtMHZPUUVaTWo5bWc?oc=5</t>
-  </si>
-  <si>
-    <t>Unlocking Finance for Nature-based Solutions in Indian Cities - Climate Policy Initiative</t>
-  </si>
-  <si>
-    <t>Unlocking Finance for Nature-based Solutions in Indian Cities  Climate Policy Initiative</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNbE9VZDZKVktsajJEVG0yM1ZfWEJ3Ums3RHRTM0FOZTFEZnFwa1NFSXBSbXpLMUpzNUktWGtqSzRVN052RllQUDNMY2x3TWlFSnNUS2VyNzF5X05ZWmx1MTlYSVlwOS05WDhjcmpCZTBacHc1Q29Ba2lZUkVuclMtaFJ6ejI3Z2lkMHVYdEFJREJIdXF2ZUVXT0VMMlFaLWRoeHFKY2xMS2syRTJWZDVQaVRraTQ?oc=5</t>
-  </si>
-  <si>
-    <t>Stock market today: Dow, S&amp;P 500, Nasdaq rise as AI worries recede, with Fed minutes ahead - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Stock market today: Dow, S&amp;P 500, Nasdaq rise as AI worries recede, with Fed minutes ahead  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQcEhkYkxjdlVSbDVfTk83VmVuZ2pVTmgzNjFsRFRjc0VqelNPX1c1RFZ4am1Ra3U5TUlVWnFNTVZkTlNTRGpzanNCcUVybTlGNHNMaXR4ajc4VVZqbW55cFp5ZWJlR3NGZmM1OFEyMmFqblBQVmNwdkdLRzRSMWdfVVpwZmYyRndHczgtOHYxWTNSQ3V1WmkzcTJod0d6X0pmY3B2d0ItTmx1OWpCenVtdzUtc09PeW1JWVgwcDQxYUJIZktZRHBGTC1idnc2cFFINVE?oc=5</t>
-  </si>
-  <si>
-    <t>Snap Finance Study Finds Majority of U.S. Households Delayed Essential Purchases in 2025 as Credit Pressures Persist Into 2026 - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Snap Finance Study Finds Majority of U.S. Households Delayed Essential Purchases in 2025 as Credit Pressures Persist Into 2026  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxOTzNzdHpaNkF0TUlxNHJwdGtIRzQzdTBlNXpkUWRTbVdna1M0eE1IU1NvS1otYTAzVEFub2lvVWlKeHd6QkY3RmJ0T3NqSkVBX29Ya25DbkNydnZDRG55OGxDTksydXo4Y3JWSXNRd1U3UUY5Zm0zdlExbDVkZkxzVmxlU05Rdw?oc=5</t>
-  </si>
-  <si>
-    <t>Lightrock grabs an exit opportunity from Indian small business lender Aye Finance - ImpactAlpha</t>
-  </si>
-  <si>
-    <t>Lightrock grabs an exit opportunity from Indian small business lender Aye Finance  ImpactAlpha</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPbW5lcmJoSERuOFp0MGYzaHJXS2Q4c2FTNUgyODYybUlOZ2JKUlVLcTcwYlRoNmRxbC0tejNBZXFaSHhEaTR2Q1VDT1BEREtLWjhiM2JDSFFpM2JGMUYyazI4a2ZkTm9Ja2pCRmNtcGhqTlJzcFowVlNKWmxtOHpSR1g1X1hEaXZyVXB1Y0ZlYVlkV3N3VTVTT2U3Y1ZKMHE2VkNSeHpKNWYtUQ?oc=5</t>
-  </si>
-  <si>
-    <t>OPENLANE, Inc. Reports 2025 Financial Results - PR Newswire</t>
-  </si>
-  <si>
-    <t>OPENLANE, Inc. Reports 2025 Financial Results  PR Newswire</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNZ3FFQzNzUG81QkNjTDgycHBKSUh3NURtVi1WUkR0cGFoODg3LUFyX25YYjVYNFIzU0U2cW9YT2pkcUNxTnpWb2VoUFpGTGI2N2I0Y2tmZ1hwWVlQRzhNVU1LdnBzYkx6QUpKSlRLQmJiMHFuV0NSNkhpTEZpVTIxeTRwVmUxc2c3S01fYnVWZVJDR2Z3VzlvV2MweUw0bXJk?oc=5</t>
-  </si>
-  <si>
-    <t>Are Finance Stocks Lagging Barclays (BCS) This Year? - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Are Finance Stocks Lagging Barclays (BCS) This Year?  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPbkt4OTRYNGtDSjRKUTF5Y3hVZ242YzN0Nmlub0kzMl9KbnRRU00tMHdLVEl3aTY0V0Y5QWFzRDAtQ0M5WlVGV3ZxV1NzN3VpaWt2UVhVNWZVTDlScHA1bzg5TFlpN2p4Q0FGbHVhVVNuaWNzOTVQMTVoeklfR1hOT3h0R1ZlYmpQ?oc=5</t>
-  </si>
-  <si>
-    <t>West Virginia Senate Finance Committee approves appropriations bill for Hancock County Schools - News and Sentinel</t>
-  </si>
-  <si>
-    <t>West Virginia Senate Finance Committee approves appropriations bill for Hancock County Schools  News and Sentinel</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxORmNQWEtJSnc0OEQ2Yl92TldtMHJrVEdaZUdNdHNvb0pWdmpLcGdTV0xXZE5EcmJsWWFLSmxaOENUdUFqel92bTRjZ1g0TU9uLXVHTXNTY2x0VmVYV1Y4V1p4RTZKVDVNUGZHY0l3V3dWdmtuVGxMcmtOQVpralpLaDdGNXJ6OUt6dEpsMlNHQzNSOXpsclJBX1lOMXYzdkptaGlJRkRhNVdIaWowc2pFTTM5VlRFVlJsM0FCaU81TDl0by1fVVRCcUhYdThWYUdJbVRwUElna0hEVjQtM0NhYUlBcUtBUQ?oc=5</t>
+    <t>JPMorgan names Catherine O'Donnell head of North America Leveraged Finance - Reuters</t>
+  </si>
+  <si>
+    <t>JPMorgan names Catherine O'Donnell head of North America Leveraged Finance  Reuters</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOWEpseFJwUG1ZQno2N1VKRENxaUhBQjIyWDRwTHZSVXJmWGNndkF6dkxITFJkMENyb3NVMjRwaXRPOTd1TnU1LTNXdzdWTk55Tmk0b1ZzUG5RdzBEbGJWbXFOY2hfaHl2QldMdUF6RmhfdGVqMXhibk03cGNXVmVZaDVMUm92N0d5WWZkVHFuc254cGpMSG5SOXVBRnpNLVQyRWE3MjNxTlFvY1dkbkIzb2ZmSlk1eDZrb0VkRUpQcmQ?oc=5</t>
+  </si>
+  <si>
+    <t>Will investors buy the transition bond label? - Environmental Finance</t>
+  </si>
+  <si>
+    <t>Will investors buy the transition bond label?  Environmental Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOaFF0YzF2bWd3eHM4WHR5NHVzSlNRNTFUYk1QLWxCbjd6V2dzRkxHU2ttOGxsV1ZPVEtxTnBscVNLYjFYNGtEUGhIRzNaMUNUVGxaZkkwY2hOd1V2VVN0Y1RfM21SYXdnUlJtdktzWDkxN0JVTU41c0xuOTFrTFM2LU1jellYOTNaTGh6NGJhOWpXSFRxUnZZcG12Q3pVZV9sSHU0TnBGYw?oc=5</t>
+  </si>
+  <si>
+    <t>Gator Capital Management’s Investment Thesis for TFS Financial Corporation (TFSL) - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Gator Capital Management’s Investment Thesis for TFS Financial Corporation (TFSL)  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQQVpxUHI5eVNWd1FLVmJEdmtqbFd4Y2FfenVZbnNyVGdIWjJKM3VBUURxSVVRMi1tQjJPUWVaX2d2N051QVpqV2kzb05TdFRPcWpyejNKWDExUVRQUjFBX280MGRuM3BhZjNwYXR0N0pwOFlzN3RFRTQyM3dFRVdnVFdIMGZrMWFWSUY5YWs5dkJqdw?oc=5</t>
+  </si>
+  <si>
+    <t>Stock market today: Dow, S&amp;P 500, Nasdaq futures rise as AI worries recede, with Fed minutes ahead - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Stock market today: Dow, S&amp;P 500, Nasdaq futures rise as AI worries recede, with Fed minutes ahead  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQQWYwUXZORzFQZ1lfcUhPRnZVODdGLTdXbWRtVjVCVXRaV0dRQ2ktQmVYUXhDV0hULXFBclcyeDcyc0FuamRGdkI3SDRHYlFSa1JNa1NDSzM0engwclZWTnBqZmNYa0stRl9vcllHQ2E5cEZBc0hveVZ6M2MtLVBLTC0zaV9uWEVRYnpCemYwSUxuYlNiZ0VhRXl2c2RQblIyY0xFY2h6WElsbFJ5LXZaVUtpN09yRS1uTm9PTEFVQTRjSW5iNDNWMUVFRkhiNl9USXRyYV9BRVpiZ1ll?oc=5</t>
+  </si>
+  <si>
+    <t>Finance Chair Warns of Prediction Market Impact on Sports Gaming - State Affairs</t>
+  </si>
+  <si>
+    <t>Finance Chair Warns of Prediction Market Impact on Sports Gaming  State Affairs</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE04U3ZjVE9SNjRpN0hGSkEyNUNqdWMwclFieHV0UlpZNHdGRV9lSmdrdVlhcnVaSHJmQ3lpb3J6YnBnS2p2VEN4R0xwMjJ0d2NkNURTNFNpdzFOZ2xPTmppdGFxOFNJQTh2WHFFRTNxeGY1YkpXX01sWTJOUVBUNkE?oc=5</t>
+  </si>
+  <si>
+    <t>Medicare Advantage growth slows - Healthcare Finance News</t>
+  </si>
+  <si>
+    <t>Medicare Advantage growth slows  Healthcare Finance News</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5pQnk4Q0VjOEViR3Uyc29jUVota3pxNjFkOHVDOXJYX0RzNjA4TWxVVkd2NnRFU09oelViOGVjM2laRkFKRHREN2tId3lOWWM3TVVzeXd2Q0dBSTBvcnFua0JWYm9ibzY4aDVVTzgtQVBvVW9fWjh6cVVLWXhrWjg?oc=5</t>
+  </si>
+  <si>
+    <t>Morning Bid: Changing of Lagarde - Reuters</t>
+  </si>
+  <si>
+    <t>Morning Bid: Changing of Lagarde  Reuters</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPbExHYkdzZWlmeWtDWkJaVGtsV2ptaFRRT0tkT2l1cW9FMDN1NXNHdmoyWEFkN0JPakhxX2l1WFVWMlJ3M3NBNFplM2dwZC16OEl0MjdzYWVMcXlObGJMT2RsTExOaGNYUXZoVkVzcVZpUWR4V3VFYjFnb1NkSEFEUERB?oc=5</t>
   </si>
   <si>
     <t>Analog Devices Reports Fiscal First Quarter 2026 Financial Results - PR Newswire</t>
@@ -1961,40 +2042,49 @@
     <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPdk5GakFqU2s3RjN1N0VIb3RsZ0ZPQ1NqRVFXZXMtZ1QtV1AxWUxzWjVDemJrQmppMm9WTWZyMk5COVRDUF9WWk9zalhYamlIaUZOMlRVMTF6SUNJMnJRWEFZQ2hEeUVXb0dRNUpsdk9ydmxEVXlVcW9OdUhQX2VmNFpyZkJvQWdob0h4VzlWMGJKWTFUVTJySXZ0NGhJdmp1SWdVSGZLUkoxaFVfMEJoTG43QzZuYTlkTXRsNF9NWQ?oc=5</t>
   </si>
   <si>
-    <t>Financial scams are on the rise — but what’s being done about it? - The Hill</t>
-  </si>
-  <si>
-    <t>Financial scams are on the rise — but what’s being done about it?  The Hill</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQbFU0OFZxQ2tVdlpqamVrdldYbTE1N0NkOWw4RjlnQ3lDaFVIanpfTFNrbllSVWMySl9DS0FmZzlWSDRCTEloTEF2Vms5QmRPaFpJcjM0T3RTa3JtY3UtbW1tVlpHQkxYYWRlTTI4NWMwaXp2SVdYZDdZUlRYMHV4RmVXWdIBiAFBVV95cUxOZ1ZOWTllSWJKWEFaLTl4ZEk4LUx5dzl3M2tiMEhKZWhLb0dpaW16QnJ3RzRudExGS2NPeGZjYVVBbnItVGxfNE1pWUxyZG1SMmMxSEdxSVhIZndmM0FpRDdTbFFrNHluWVh6a2M5T3RRT2FsdkdJdlhJaGc1WXp1dVNFNXhlQ2hI?oc=5</t>
-  </si>
-  <si>
-    <t>JPMorgan names Catherine O'Donnell head of North America Leveraged Finance - Reuters</t>
-  </si>
-  <si>
-    <t>JPMorgan names Catherine O'Donnell head of North America Leveraged Finance  Reuters</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOWEpseFJwUG1ZQno2N1VKRENxaUhBQjIyWDRwTHZSVXJmWGNndkF6dkxITFJkMENyb3NVMjRwaXRPOTd1TnU1LTNXdzdWTk55Tmk0b1ZzUG5RdzBEbGJWbXFOY2hfaHl2QldMdUF6RmhfdGVqMXhibk03cGNXVmVZaDVMUm92N0d5WWZkVHFuc254cGpMSG5SOXVBRnpNLVQyRWE3MjNxTlFvY1dkbkIzb2ZmSlk1eDZrb0VkRUpQcmQ?oc=5</t>
-  </si>
-  <si>
-    <t>Will investors buy the transition bond label? - Environmental Finance</t>
-  </si>
-  <si>
-    <t>Will investors buy the transition bond label?  Environmental Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOaFF0YzF2bWd3eHM4WHR5NHVzSlNRNTFUYk1QLWxCbjd6V2dzRkxHU2ttOGxsV1ZPVEtxTnBscVNLYjFYNGtEUGhIRzNaMUNUVGxaZkkwY2hOd1V2VVN0Y1RfM21SYXdnUlJtdktzWDkxN0JVTU41c0xuOTFrTFM2LU1jellYOTNaTGh6NGJhOWpXSFRxUnZZcG12Q3pVZV9sSHU0TnBGYw?oc=5</t>
-  </si>
-  <si>
-    <t>Gator Capital Management’s Investment Thesis for TFS Financial Corporation (TFSL) - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Gator Capital Management’s Investment Thesis for TFS Financial Corporation (TFSL)  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQQVpxUHI5eVNWd1FLVmJEdmtqbFd4Y2FfenVZbnNyVGdIWjJKM3VBUURxSVVRMi1tQjJPUWVaX2d2N051QVpqV2kzb05TdFRPcWpyejNKWDExUVRQUjFBX280MGRuM3BhZjNwYXR0N0pwOFlzN3RFRTQyM3dFRVdnVFdIMGZrMWFWSUY5YWs5dkJqdw?oc=5</t>
+    <t>Gorilla Technology Acquires Shackleton Finance to Establish Regulated Capital Platform and Fund AI Infrastructure Growth - Investing News Network</t>
+  </si>
+  <si>
+    <t>Gorilla Technology Acquires Shackleton Finance to Establish Regulated Capital Platform and Fund AI Infrastructure Growth  Investing News Network</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPNmZQaXZmQVBnOURjeVFnZ2Y4U3U2MU1LVHRQUTdMLTUyWXFvM2htN3RJaVQwQmU2M203N2x1SkYwNVhtZnZ3QXNqNDZEVzU5N1pmTUhMX096M1ZhMUd2U2p6VXNrMWNnX092TEhMVUNQbWlua0JOc1hFYkNST1BzZ2E4cW95TVhCSDltX2xZeXJYUzY3Q0JZckxMUkQzUUhVX2tVc1YxbDg2WWhZWXd2YkctWEd1ME5qbGcyY1RTYl9tcWFSVHZUOWdtZTl3SkZoWU42WlRuTm9rWlRRZG8zaw?oc=5</t>
+  </si>
+  <si>
+    <t>Tuition, financial aid rates set for 2026–27 academic year - University of Rochester</t>
+  </si>
+  <si>
+    <t>Tuition, financial aid rates set for 2026–27 academic year  University of Rochester</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNclRRcDI0YUNSbzR1aWhpc29FZVBtT0ZZTlkxRXpkdjUyZXJfN0NBSTZjaFJLeDIxbHFNS2J0NWN6QURmZDI5OWg1NHdSYzVzTlhzbDM2R0gwVzNiXzJkWlpjcTlQNVBNOGpFc1BSbTRVQm81V0dfeDRQZzRJRzFNdmNKT3A5OC1qclB5dkxCaWNBOWpWZlBCOFFncw?oc=5</t>
+  </si>
+  <si>
+    <t>Sheffield Financial, Mercury Marine launch financing partnership for outboard engines and boat packages - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Sheffield Financial, Mercury Marine launch financing partnership for outboard engines and boat packages  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNRDdXZFRmVHVSYUxLME9OTWN2R0g0TDFDR2ptUl80UmZmNVlyVkZPTWkyTmotTXBja2NqLUVxdk1EWnFucU51d3F3UlZTWTlydy1TNVFRa0lfX1hnT3YwMXNyQldaVEphSHpYSFNBYjlPcmJCcGxVdDhKSUZBX0NVY0Z6UnFVMzhUcTJXNlVyNUM?oc=5</t>
+  </si>
+  <si>
+    <t>UK's YouGov appoints former ITV finance chief as chair - Reuters</t>
+  </si>
+  <si>
+    <t>UK's YouGov appoints former ITV finance chief as chair  Reuters</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNUldhNkVfU0otcmZKSGRkQU8waHdmWnpUQVIzTzQwOHBsejlIdEFjenVGWDh4YmZsMXcycTZNbTVLdzFkMF8xZlBrUE5UMHgzYURabUFtRHFQWHhTTXBHa3pYcjhGMzVoZUlyZVZ4WE9WU3o5TjdzTHhIME05S0JRR05DRjNuMFBZajlLSV9lbEZIbk5CZTBpaGVn?oc=5</t>
+  </si>
+  <si>
+    <t>Four health systems deploy AI to control spend - Healthcare Finance News</t>
+  </si>
+  <si>
+    <t>Four health systems deploy AI to control spend  Healthcare Finance News</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNc1kycHlPNTVqbVNZY0dFNjlfem0zamM5cDVhWjNmc3FSc0ZNcUVQMmlfODJnUVF2S3hsOUV6N1REUDYxMXZwY2diRkhlY0thSmFKZVpEeUZ0ZWE3cFU5dDJEZGhXQ2poc0VlU2RSbXFlM3Q0cW9WUnhfTmFKdzhZeHBOWGd0S3dUUHVVa09NYw?oc=5</t>
   </si>
   <si>
     <t>2026 Africa SABRE Awards: African Development Bank’s access-to-finance “AFAWA: Banking on Women” communications wins top global campaign honors - African Development Bank Group</t>
@@ -2006,60 +2096,6 @@
     <t>https://news.google.com/rss/articles/CBMingJBVV95cUxPNFVQU1NQV2VGeEtVMWFlUHRTa1ByUFUxV29fZ255Xzk3eUR2UUJpVWJuU2xGd09JYTlWaWM5ejZza00wM19QMWZSYjU3THlVSGoyU0ZXdGRpYktEeXJOMzZ2N2VkblZZQjd3emkxU2l6eVJ1amdabGlwelhlVE9fUUhhM1N0MEJaUXJsRVg5WGVpeHlDRGJyLWZiSXkzWk94OWxBRTdrYlJhdUdvT0dmalZka1FTT0FGb293dlo2M2kyZ0psR3NDbDM4SXRSZUFRb3c2NGJlbzhxMk1vckFnZlhwMjF1WkFMc0djc01kd2h4eFZ5dG5uZUx0ekFKR3FBbzJucHI5R0pMQjYySTJkUEVGNTR5cGplOVQ4WUJn?oc=5</t>
   </si>
   <si>
-    <t>Tuition, financial aid rates set for 2026–27 academic year - University of Rochester</t>
-  </si>
-  <si>
-    <t>Tuition, financial aid rates set for 2026–27 academic year  University of Rochester</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNclRRcDI0YUNSbzR1aWhpc29FZVBtT0ZZTlkxRXpkdjUyZXJfN0NBSTZjaFJLeDIxbHFNS2J0NWN6QURmZDI5OWg1NHdSYzVzTlhzbDM2R0gwVzNiXzJkWlpjcTlQNVBNOGpFc1BSbTRVQm81V0dfeDRQZzRJRzFNdmNKT3A5OC1qclB5dkxCaWNBOWpWZlBCOFFncw?oc=5</t>
-  </si>
-  <si>
-    <t>Gorilla Technology Acquires Shackleton Finance to Establish Regulated Capital Platform and Fund AI Infrastructure Growth - Investing News Network</t>
-  </si>
-  <si>
-    <t>Gorilla Technology Acquires Shackleton Finance to Establish Regulated Capital Platform and Fund AI Infrastructure Growth  Investing News Network</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPNmZQaXZmQVBnOURjeVFnZ2Y4U3U2MU1LVHRQUTdMLTUyWXFvM2htN3RJaVQwQmU2M203N2x1SkYwNVhtZnZ3QXNqNDZEVzU5N1pmTUhMX096M1ZhMUd2U2p6VXNrMWNnX092TEhMVUNQbWlua0JOc1hFYkNST1BzZ2E4cW95TVhCSDltX2xZeXJYUzY3Q0JZckxMUkQzUUhVX2tVc1YxbDg2WWhZWXd2YkctWEd1ME5qbGcyY1RTYl9tcWFSVHZUOWdtZTl3SkZoWU42WlRuTm9rWlRRZG8zaw?oc=5</t>
-  </si>
-  <si>
-    <t>Stock market today: Dow, S&amp;P 500, Nasdaq futures rise as AI worries recede, with Fed minutes ahead - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Stock market today: Dow, S&amp;P 500, Nasdaq futures rise as AI worries recede, with Fed minutes ahead  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQQWYwUXZORzFQZ1lfcUhPRnZVODdGLTdXbWRtVjVCVXRaV0dRQ2ktQmVYUXhDV0hULXFBclcyeDcyc0FuamRGdkI3SDRHYlFSa1JNa1NDSzM0engwclZWTnBqZmNYa0stRl9vcllHQ2E5cEZBc0hveVZ6M2MtLVBLTC0zaV9uWEVRYnpCemYwSUxuYlNiZ0VhRXl2c2RQblIyY0xFY2h6WElsbFJ5LXZaVUtpN09yRS1uTm9PTEFVQTRjSW5iNDNWMUVFRkhiNl9USXRyYV9BRVpiZ1ll?oc=5</t>
-  </si>
-  <si>
-    <t>Finance Chair Warns of Prediction Market Impact on Sports Gaming - State Affairs</t>
-  </si>
-  <si>
-    <t>Finance Chair Warns of Prediction Market Impact on Sports Gaming  State Affairs</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE04U3ZjVE9SNjRpN0hGSkEyNUNqdWMwclFieHV0UlpZNHdGRV9lSmdrdVlhcnVaSHJmQ3lpb3J6YnBnS2p2VEN4R0xwMjJ0d2NkNURTNFNpdzFOZ2xPTmppdGFxOFNJQTh2WHFFRTNxeGY1YkpXX01sWTJOUVBUNkE?oc=5</t>
-  </si>
-  <si>
-    <t>Morning Bid: Changing of Lagarde - Reuters</t>
-  </si>
-  <si>
-    <t>Morning Bid: Changing of Lagarde  Reuters</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPbExHYkdzZWlmeWtDWkJaVGtsV2ptaFRRT0tkT2l1cW9FMDN1NXNHdmoyWEFkN0JPakhxX2l1WFVWMlJ3M3NBNFplM2dwZC16OEl0MjdzYWVMcXlObGJMT2RsTExOaGNYUXZoVkVzcVZpUWR4V3VFYjFnb1NkSEFEUERB?oc=5</t>
-  </si>
-  <si>
-    <t>Medicare Advantage growth slows - Healthcare Finance News</t>
-  </si>
-  <si>
-    <t>Medicare Advantage growth slows  Healthcare Finance News</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5pQnk4Q0VjOEViR3Uyc29jUVota3pxNjFkOHVDOXJYX0RzNjA4TWxVVkd2NnRFU09oelViOGVjM2laRkFKRHREN2tId3lOWWM3TVVzeXd2Q0dBSTBvcnFua0JWYm9ibzY4aDVVTzgtQVBvVW9fWjh6cVVLWXhrWjg?oc=5</t>
-  </si>
-  <si>
     <t>Let Idaho fix campaign finance, get dark money out of politics | Opinion - Idaho Statesman</t>
   </si>
   <si>
@@ -2069,6 +2105,42 @@
     <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNWnMya0FLQWJQdFdvYVlfT3EzLXFsMFFoQU83OVdmMDI4ZlVmbTNjd0ZXeXBfWGN0VlZVdE9PZWVYZms3c3p6QUp6ZlZoOE9pdHFGaFZFN3lJazlxeWppOEpkN2ZiVUI2TDRadHhuc0dCRy1DekFmOEdRVnkySDdtcU5B0gGCAUFVX3lxTE42d2trUFl6Ql9PYjh6MFhsaU1KS1BQc2ZwWnZkTnRrX3pIbTJoc0czaHUweGVsVHRNSmNZX1ZMZ3hqeXpRdGJKb3RaUVAwRlB2VjZGVmJ0Wmh6LWMzQzdnOWFPbDV3cDhNX3pvV0tSVXZtRXNTOGVYbVYxbGRpbUxJZmc?oc=5</t>
   </si>
   <si>
+    <t>Senate bill decreasing campaign finance transparency passed - theintermountain.com</t>
+  </si>
+  <si>
+    <t>Senate bill decreasing campaign finance transparency passed  theintermountain.com</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcVJRNTA1YVFuTldWNjFfNnV2bV9wYS1UNHR2UWszUEQ2NlNlRjRGaEFIS3NoQ3c3UExHVmF4UHFZeThYQUgtSURkN1ZPV1hBRUx5RndTV2VqT3JzQTVvc1NyOHpINnAxQS1zLWJHMlBLLXVSSGQ3TXd0ZHJoblhSWlFfMWFhaXhaRTRWR25vdkJhVURNaGtDX29MNjJfWFQtbXhWTFBkVXhUdnhYcENsZl9VNlFCaTIx?oc=5</t>
+  </si>
+  <si>
+    <t>Xerox partners with Texas PE firm, secures $450M in financing - Hartford Business Journal</t>
+  </si>
+  <si>
+    <t>Xerox partners with Texas PE firm, secures $450M in financing  Hartford Business Journal</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQSDFpZ0hmb213MU02blo3Rk9nU3phencxblN0YnBvTW5kZEtDN1gzdWtEaU5nc2pyNmFUYjNTM1VaRDVOSGNZMF9kUEQ0Z1F3cVVsczlkaEw2RkhFSnhLSXVwbHREcEZCUUFJbXpiT3dEN2plOU5tOTZBTVRMNmNoNXNzQ1VlOHEtdFpUMUNGZE9SN083cXFfaUk2Z3cwZw?oc=5</t>
+  </si>
+  <si>
+    <t>Embedded Finance Reshapes SME Cash-Flow Stability: Implications For Advisors - Wealth Briefing</t>
+  </si>
+  <si>
+    <t>Embedded Finance Reshapes SME Cash-Flow Stability: Implications For Advisors  Wealth Briefing</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOcFNnTkg3WGFKSWI3c2toU0RhTmJzdHNyVndiOW5sSDVyaWVqVkZkQ2FqMEREUWVsWFhWUXVZdGdBNEZXYUV5WmxtSE1YOVVEZTRaY2pEanFtczNXOTN2NFNmeWhkSlFSRGVfc2YxcGllVFFYaXgxVnA2cFctbGs3ei1USEFtM042eGZqeE0xS0dmY1ZaUkZKRy1fcmNUWkxyVFNhUlN6RTA0N3cwRW9FYUM2QXprMTUwd2tVRGJERnZrRng1VmJYYmJvX0h3dw?oc=5</t>
+  </si>
+  <si>
+    <t>Japan Election Supermajority Boosts Market Confidence In Economic Recovery - Global Finance Magazine</t>
+  </si>
+  <si>
+    <t>Japan Election Supermajority Boosts Market Confidence In Economic Recovery  Global Finance Magazine</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPenFOalRHdHhVR2dmNUR4SDhSeEVzLU1ZLUVYUk1UMXZwNGgtTWI4REJISU90TlhIeXRHaEtRY19RalVwSXNjUE9zUXBWNUFsbTZEQURudWE4WmpQOTdFNE9MUkZFMlFDcFg3NkVBQnk1a21UMF9tR0dXcV9DM0trOTZtSF96YTNHMm43U1VvUUlrNTE0cGN5UWwwZU15T1Q1TlZJQ3pyRTA3eHAxZ1NuWWZVX3VFcVM1UlJOY1VR?oc=5</t>
+  </si>
+  <si>
     <t>Symposium on International Investment Law &amp; Contemporary Crises: Divergent Approaches to the Nationality of Corporate Claimants in Banking and Finance Investor-State Arbitration - Opinio Juris</t>
   </si>
   <si>
@@ -2078,67 +2150,85 @@
     <t>https://news.google.com/rss/articles/CBMiswJBVV95cUxOVzVCTXM1OXlwdTg3WG1qR1poQW00WjBXeFhtNF9IMEhhWEZKbTBtV0lEUFNUWURScUFPVzFjOEQtMFQycnJmTmlUTFZaZm52X055djVCNDlxT1lEQXRuTnQ2Zk9iVEtLSHJiWEI2SkpsTmVCOUx3dlJkUERIcWNpMHF1WWpKeVJuMDI3bC1kZ0p1RnFuZzdoZlpqY2pVQkJTbGtqT2FpRkh4OGZqLUJJaDBCQzNTdmIxLS1mdnJ3T3pCOXZ0dGlwa0hRYTNDUXIyOFVsZjNycV9wT0tsTlhpTFRZWG5FazRaWVRzcjFaYXlYRUxEV1BnQi1jdDVqZzF1ZXQwdXdsS1pVRzQ5bnN5VTFyQVBKV05YYlFOUlZFV095TDJpOW9INEZQLXo0UXgzRnVN?oc=5</t>
   </si>
   <si>
-    <t>Sheffield Financial, Mercury Marine launch financing partnership for outboard engines and boat packages - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Sheffield Financial, Mercury Marine launch financing partnership for outboard engines and boat packages  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNRDdXZFRmVHVSYUxLME9OTWN2R0g0TDFDR2ptUl80UmZmNVlyVkZPTWkyTmotTXBja2NqLUVxdk1EWnFucU51d3F3UlZTWTlydy1TNVFRa0lfX1hnT3YwMXNyQldaVEphSHpYSFNBYjlPcmJCcGxVdDhKSUZBX0NVY0Z6UnFVMzhUcTJXNlVyNUM?oc=5</t>
-  </si>
-  <si>
-    <t>UK's YouGov appoints former ITV finance chief as chair - Reuters</t>
-  </si>
-  <si>
-    <t>UK's YouGov appoints former ITV finance chief as chair  Reuters</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNUldhNkVfU0otcmZKSGRkQU8waHdmWnpUQVIzTzQwOHBsejlIdEFjenVGWDh4YmZsMXcycTZNbTVLdzFkMF8xZlBrUE5UMHgzYURabUFtRHFQWHhTTXBHa3pYcjhGMzVoZUlyZVZ4WE9WU3o5TjdzTHhIME05S0JRR05DRjNuMFBZajlLSV9lbEZIbk5CZTBpaGVn?oc=5</t>
-  </si>
-  <si>
-    <t>Four health systems deploy AI to control spend - Healthcare Finance News</t>
-  </si>
-  <si>
-    <t>Four health systems deploy AI to control spend  Healthcare Finance News</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNc1kycHlPNTVqbVNZY0dFNjlfem0zamM5cDVhWjNmc3FSc0ZNcUVQMmlfODJnUVF2S3hsOUV6N1REUDYxMXZwY2diRkhlY0thSmFKZVpEeUZ0ZWE3cFU5dDJEZGhXQ2poc0VlU2RSbXFlM3Q0cW9WUnhfTmFKdzhZeHBOWGd0S3dUUHVVa09NYw?oc=5</t>
-  </si>
-  <si>
-    <t>Senate bill decreasing campaign finance transparency passed - theintermountain.com</t>
-  </si>
-  <si>
-    <t>Senate bill decreasing campaign finance transparency passed  theintermountain.com</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNcVJRNTA1YVFuTldWNjFfNnV2bV9wYS1UNHR2UWszUEQ2NlNlRjRGaEFIS3NoQ3c3UExHVmF4UHFZeThYQUgtSURkN1ZPV1hBRUx5RndTV2VqT3JzQTVvc1NyOHpINnAxQS1zLWJHMlBLLXVSSGQ3TXd0ZHJoblhSWlFfMWFhaXhaRTRWR25vdkJhVURNaGtDX29MNjJfWFQtbXhWTFBkVXhUdnhYcENsZl9VNlFCaTIx?oc=5</t>
-  </si>
-  <si>
-    <t>Xerox partners with Texas PE firm, secures $450M in financing - Hartford Business Journal</t>
-  </si>
-  <si>
-    <t>Xerox partners with Texas PE firm, secures $450M in financing  Hartford Business Journal</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQSDFpZ0hmb213MU02blo3Rk9nU3phencxblN0YnBvTW5kZEtDN1gzdWtEaU5nc2pyNmFUYjNTM1VaRDVOSGNZMF9kUEQ0Z1F3cVVsczlkaEw2RkhFSnhLSXVwbHREcEZCUUFJbXpiT3dEN2plOU5tOTZBTVRMNmNoNXNzQ1VlOHEtdFpUMUNGZE9SN083cXFfaUk2Z3cwZw?oc=5</t>
-  </si>
-  <si>
-    <t>Japan Election Supermajority Boosts Market Confidence In Economic Recovery - Global Finance Magazine</t>
-  </si>
-  <si>
-    <t>Japan Election Supermajority Boosts Market Confidence In Economic Recovery  Global Finance Magazine</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPenFOalRHdHhVR2dmNUR4SDhSeEVzLU1ZLUVYUk1UMXZwNGgtTWI4REJISU90TlhIeXRHaEtRY19RalVwSXNjUE9zUXBWNUFsbTZEQURudWE4WmpQOTdFNE9MUkZFMlFDcFg3NkVBQnk1a21UMF9tR0dXcV9DM0trOTZtSF96YTNHMm43U1VvUUlrNTE0cGN5UWwwZU15T1Q1TlZJQ3pyRTA3eHAxZ1NuWWZVX3VFcVM1UlJOY1VR?oc=5</t>
-  </si>
-  <si>
-    <t>Embedded Finance Reshapes SME Cash-Flow Stability: Implications For Advisors - Wealth Briefing</t>
-  </si>
-  <si>
-    <t>Embedded Finance Reshapes SME Cash-Flow Stability: Implications For Advisors  Wealth Briefing</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOcFNnTkg3WGFKSWI3c2toU0RhTmJzdHNyVndiOW5sSDVyaWVqVkZkQ2FqMEREUWVsWFhWUXVZdGdBNEZXYUV5WmxtSE1YOVVEZTRaY2pEanFtczNXOTN2NFNmeWhkSlFSRGVfc2YxcGllVFFYaXgxVnA2cFctbGs3ei1USEFtM042eGZqeE0xS0dmY1ZaUkZKRy1fcmNUWkxyVFNhUlN6RTA0N3cwRW9FYUM2QXprMTUwd2tVRGJERnZrRng1VmJYYmJvX0h3dw?oc=5</t>
+    <t>Stock market today: Dow, S&amp;P 500, Nasdaq futures climb with AI disruption in focus, Fed minutes ahead - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Stock market today: Dow, S&amp;P 500, Nasdaq futures climb with AI disruption in focus, Fed minutes ahead  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxNM2lKWUJWMWdzZExXazVwM3M0Y0w5WnBKYUI1SHZWSDNnSkgxUVgxSUNVOEpneDh6NFNPdS1PZDJVWWhLbndnMWk4bFNUS3ZOWVJQVUpTTldhcUdEdmxDeTRDaS1hVURCUmgtR2RBb3d2TDBYbGVLUk5zZUl3cHQ5MmhiRkk0WTF6YXZZeXEtdG9EcF92Qlg3ang3TTFZMElfRWRQamFaRGdrcG5Ta3I0OHVPTGNMc3o3Q0F4Y1k0VVk4a2o5NEd1Y1lTQ0xkdVpNNlIyUU5uamZNZmJNREtLcA?oc=5</t>
+  </si>
+  <si>
+    <t>red violet to Announce Fourth Quarter and Full Year 2025 Financial Results on March 4, 2026 - Yahoo Finance UK</t>
+  </si>
+  <si>
+    <t>red violet to Announce Fourth Quarter and Full Year 2025 Financial Results on March 4, 2026  Yahoo Finance UK</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNUmpwMW1xVEFBUWZjcWRMRG1VVjRZTDFYT1pvQ3NqLVM0ZlQyX2pCc1ZyVHNQWGpaaTVUVVd2NHNMWHhXRmRQREVoWFJlZmg0Z25Yc29mNzFiU1AzR2U1N2swWWJ3S093Z21fV2d0VTlQTUtuUXlGMFJEa3VCNU5veWRTMmxxUkFRLU5N?oc=5</t>
+  </si>
+  <si>
+    <t>Commentary: Campaign finance reform suffers the risk of ‘a deal that has yet to be real - The Portland Tribune</t>
+  </si>
+  <si>
+    <t>Commentary: Campaign finance reform suffers the risk of ‘a deal that has yet to be real  The Portland Tribune</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxNUWZMLXk4dms5VEh5YWJIMVZLSVdjOGExcXRQZEFhSDAzQ0d3WXRrYVhraXVDUXkyQjV4NnhQNUJxUlN0cTFRRGVORDNjOU9hS2NOZ2VMZ2NSY2w0YzRsMFQyZWJYQWJNZFNnakdvX0NZbTdjaFlSQ0dvc2dIZExUc0ctWHNGVU42QmpTcmVMblJLcE9KNlhCQTczUlJrU0JTWF93aF9OczVOcUhKSU0wVHd5bk1vSm1zS2l4S2VPMkI2OEE?oc=5</t>
+  </si>
+  <si>
+    <t>Top 10: AI Tools for Finance - AI Magazine</t>
+  </si>
+  <si>
+    <t>Top 10: AI Tools for Finance  AI Magazine</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBMangwQjkyOTJGb2d1SDI0U1N6M2o2cERWekxqbmlWT2FrZ3gtcU5ROElabGIxTjM5eEUwb2JpR09VS1UwQjAtYXFCUHEyTDU3VVdNNmtaUkxCdVdyaC1TUmVaVWNqNFU?oc=5</t>
+  </si>
+  <si>
+    <t>Pasinex Announces Q4 2025 Financial Results - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Pasinex Announces Q4 2025 Financial Results  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPVDJNaFBkZHlKN0g4QV9DRmRlZUdHSHVHbkdXYUxiYmJmRV96SFlJWEFoNEY4NFRMX2NxZ29peVh6dG9PSVpNN1cwa0xiSGVQYnp6cFdlbE1aMDhMc0lnckkwbUJCcGVJM3RQcEhHbFRpWlpGcllPU0Y2bHlFYmtaVWR3R2RiMWV5?oc=5</t>
+  </si>
+  <si>
+    <t>5 Financial Transaction Stocks to Watch Despite Elevated Expense Level - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>5 Financial Transaction Stocks to Watch Despite Elevated Expense Level  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPdThLN21OaFZvSC1IZ2ZyeEdoUVc0TnQxNUJjLXdGYkJ1UGMtSDBtSFVycXFOTktWOHlScU03YjVzc1ZiWnQwSnphYWpNSHdtVVJBQTUteHlSbWtwZ3ZJOWJkODl6NnBwd1JtaU0wdExoX0JQTjNKd3BLcHN4R1NtNC03VDBJTlpVcmc?oc=5</t>
+  </si>
+  <si>
+    <t>Financial &amp; Tax Information - Crescent Energy</t>
+  </si>
+  <si>
+    <t>Financial &amp; Tax Information  Crescent Energy</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOT2QzcEFjdlE0Ujd1TE1tUWtXZXhPajJkSkJBcUNaVHBaSTJSV0xZamFUd0UydjBPSC1waDAzNUd0dTQ0c2lHeEM5YTRoUGxFQ0JIUGFrTU51UUpTNzVoYXUyNDR0RzVGR202WHY5QkdRRjh0N0hVbFVqNjVpRVdTR3RScEJZRnZVVThyRk9YRW5GUmQxVXVaLXhudw?oc=5</t>
+  </si>
+  <si>
+    <t>Moderna stock surges as FDA reverses course, agrees to review new flu shot - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Moderna stock surges as FDA reverses course, agrees to review new flu shot  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQZ0t2N0F6U19YUjNIcE5WeGE0Ukt5VjZYSlRjWUNpd25HRnZpV0l0Mnd4N01OU3F6THRGY3FTWWREdFYzVXhVNUJyVDBxRWRVWm9Kc3VFOGl3OWhNZXYyaUs4LW9fSnBHajRSUXhvUUsxQ1gtelZiOXNnR0pnbnlOU3EwVHFvLWdNT2NUdnY3OWlzc2tiZU9mQTZZN0I2aW9RRExXVEhuTHZhSzFySnZsWTZPeDl0eWRTVE1n?oc=5</t>
+  </si>
+  <si>
+    <t>1 Financial Stock That Could Turn $250 Per Month Into $1.4 Million - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>1 Financial Stock That Could Turn $250 Per Month Into $1.4 Million  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9LV2tVdFpfN252eWtFWGtYaFhTM1pJbk5SOGtoVUdraE90YkRuNWtxRmw5VEJHS3NGT25lRkdyeENGNFc0a3ZFZHI3NldxbF85b3BoemZPdnRXeHZRT3BHQlZIUjRIa0xsYjVXV1VMTVR6NlcwODJ4UllMREFNSTQ?oc=5</t>
   </si>
   <si>
     <t>The capex crucible: What finance teams can learn from data center builds - McKinsey &amp; Company</t>
@@ -2150,69 +2240,6 @@
     <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxNLUNwUVFROUdldVdjQ0ZwMnM5RmE5Y3BmTXo0bWhWd1Y2ZVdjbEJhSllULXRIdThRWV9rc2xURGk3V2NRcU0waWpNYXFjNGpXWlBqcm15R0RkYUdRVy1PWUFQNmVRUXVVOXJ4MXNxQlI3Yk8xZ0dvNFg2QjVKUl9PWHBLVDAzX1BicHA4dnUwazRjVE9ITkVLbWJiUjhzZGloVG0zQm1LM1ItRjlkQVVDYldCejR3Q0F3Q2RNU2x0S3dEbUJoR3N3eW5uVTZsX1RPLUVwOGExb0phbDJETG1femxFVmVpVlI3?oc=5</t>
   </si>
   <si>
-    <t>Financial &amp; Tax Information - Crescent Energy</t>
-  </si>
-  <si>
-    <t>Financial &amp; Tax Information  Crescent Energy</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOT2QzcEFjdlE0Ujd1TE1tUWtXZXhPajJkSkJBcUNaVHBaSTJSV0xZamFUd0UydjBPSC1waDAzNUd0dTQ0c2lHeEM5YTRoUGxFQ0JIUGFrTU51UUpTNzVoYXUyNDR0RzVGR202WHY5QkdRRjh0N0hVbFVqNjVpRVdTR3RScEJZRnZVVThyRk9YRW5GUmQxVXVaLXhudw?oc=5</t>
-  </si>
-  <si>
-    <t>Commentary: Campaign finance reform suffers the risk of ‘a deal that has yet to be real - The Portland Tribune</t>
-  </si>
-  <si>
-    <t>Commentary: Campaign finance reform suffers the risk of ‘a deal that has yet to be real  The Portland Tribune</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxNUWZMLXk4dms5VEh5YWJIMVZLSVdjOGExcXRQZEFhSDAzQ0d3WXRrYVhraXVDUXkyQjV4NnhQNUJxUlN0cTFRRGVORDNjOU9hS2NOZ2VMZ2NSY2w0YzRsMFQyZWJYQWJNZFNnakdvX0NZbTdjaFlSQ0dvc2dIZExUc0ctWHNGVU42QmpTcmVMblJLcE9KNlhCQTczUlJrU0JTWF93aF9OczVOcUhKSU0wVHd5bk1vSm1zS2l4S2VPMkI2OEE?oc=5</t>
-  </si>
-  <si>
-    <t>Stock market today: Dow, S&amp;P 500, Nasdaq futures climb with AI disruption in focus, Fed minutes ahead - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Stock market today: Dow, S&amp;P 500, Nasdaq futures climb with AI disruption in focus, Fed minutes ahead  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxNM2lKWUJWMWdzZExXazVwM3M0Y0w5WnBKYUI1SHZWSDNnSkgxUVgxSUNVOEpneDh6NFNPdS1PZDJVWWhLbndnMWk4bFNUS3ZOWVJQVUpTTldhcUdEdmxDeTRDaS1hVURCUmgtR2RBb3d2TDBYbGVLUk5zZUl3cHQ5MmhiRkk0WTF6YXZZeXEtdG9EcF92Qlg3ang3TTFZMElfRWRQamFaRGdrcG5Ta3I0OHVPTGNMc3o3Q0F4Y1k0VVk4a2o5NEd1Y1lTQ0xkdVpNNlIyUU5uamZNZmJNREtLcA?oc=5</t>
-  </si>
-  <si>
-    <t>red violet to Announce Fourth Quarter and Full Year 2025 Financial Results on March 4, 2026 - Yahoo Finance UK</t>
-  </si>
-  <si>
-    <t>red violet to Announce Fourth Quarter and Full Year 2025 Financial Results on March 4, 2026  Yahoo Finance UK</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNUmpwMW1xVEFBUWZjcWRMRG1VVjRZTDFYT1pvQ3NqLVM0ZlQyX2pCc1ZyVHNQWGpaaTVUVVd2NHNMWHhXRmRQREVoWFJlZmg0Z25Yc29mNzFiU1AzR2U1N2swWWJ3S093Z21fV2d0VTlQTUtuUXlGMFJEa3VCNU5veWRTMmxxUkFRLU5N?oc=5</t>
-  </si>
-  <si>
-    <t>Top 10: AI Tools for Finance - AI Magazine</t>
-  </si>
-  <si>
-    <t>Top 10: AI Tools for Finance  AI Magazine</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBMangwQjkyOTJGb2d1SDI0U1N6M2o2cERWekxqbmlWT2FrZ3gtcU5ROElabGIxTjM5eEUwb2JpR09VS1UwQjAtYXFCUHEyTDU3VVdNNmtaUkxCdVdyaC1TUmVaVWNqNFU?oc=5</t>
-  </si>
-  <si>
-    <t>Pasinex Announces Q4 2025 Financial Results - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Pasinex Announces Q4 2025 Financial Results  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPVDJNaFBkZHlKN0g4QV9DRmRlZUdHSHVHbkdXYUxiYmJmRV96SFlJWEFoNEY4NFRMX2NxZ29peVh6dG9PSVpNN1cwa0xiSGVQYnp6cFdlbE1aMDhMc0lnckkwbUJCcGVJM3RQcEhHbFRpWlpGcllPU0Y2bHlFYmtaVWR3R2RiMWV5?oc=5</t>
-  </si>
-  <si>
-    <t>5 Financial Transaction Stocks to Watch Despite Elevated Expense Level - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>5 Financial Transaction Stocks to Watch Despite Elevated Expense Level  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPdThLN21OaFZvSC1IZ2ZyeEdoUVc0TnQxNUJjLXdGYkJ1UGMtSDBtSFVycXFOTktWOHlScU03YjVzc1ZiWnQwSnphYWpNSHdtVVJBQTUteHlSbWtwZ3ZJOWJkODl6NnBwd1JtaU0wdExoX0JQTjNKd3BLcHN4R1NtNC03VDBJTlpVcmc?oc=5</t>
-  </si>
-  <si>
     <t>Papua New Guinea: 29 financial institutions decline to finance TotalEnergies liquefied natural gas project - Business and Human Rights Centre</t>
   </si>
   <si>
@@ -2222,22 +2249,58 @@
     <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxQZE11X3dpa0xGRFVUUl9XbUFULXpyc1R2N21NTTdNUlNIb0ZBSGdaVVA5YW1QbE8wMG9zd3JTakJvNDhfSkc3RXR4Z1Zkd2FfcHRDUXlwTThhLXpVV3JRaTFfSEl1alRkQ3NjeWtwakhSd2hKUlRHSjlYaWlBSUNueXJBbWV0amxycC1GOTM0aXEzMlM3M0VxNlFBZVRSRDJPdlJybDZGU1k0Tk5SbTR3VGlFN1lfOV9xSXQ1NzBzTDVNWHE4bzNXdHlvQjg2TWxaMzl5TTN2RWFmVjZrRUcyMm5KcGJNMlo3MzVfdVM3MA?oc=5</t>
   </si>
   <si>
-    <t>1 Financial Stock That Could Turn $250 Per Month Into $1.4 Million - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>1 Financial Stock That Could Turn $250 Per Month Into $1.4 Million  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9LV2tVdFpfN252eWtFWGtYaFhTM1pJbk5SOGtoVUdraE90YkRuNWtxRmw5VEJHS3NGT25lRkdyeENGNFc0a3ZFZHI3NldxbF85b3BoemZPdnRXeHZRT3BHQlZIUjRIa0xsYjVXV1VMTVR6NlcwODJ4UllMREFNSTQ?oc=5</t>
-  </si>
-  <si>
-    <t>Moderna stock surges as FDA reverses course, agrees to review new flu shot - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Moderna stock surges as FDA reverses course, agrees to review new flu shot  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQZ0t2N0F6U19YUjNIcE5WeGE0Ukt5VjZYSlRjWUNpd25HRnZpV0l0Mnd4N01OU3F6THRGY3FTWWREdFYzVXhVNUJyVDBxRWRVWm9Kc3VFOGl3OWhNZXYyaUs4LW9fSnBHajRSUXhvUUsxQ1gtelZiOXNnR0pnbnlOU3EwVHFvLWdNT2NUdnY3OWlzc2tiZU9mQTZZN0I2aW9RRExXVEhuTHZhSzFySnZsWTZPeDl0eWRTVE1n?oc=5</t>
+    <t>Gold price below $5,000 as investors wait on Fed guidance for clues - Yahoo Finance UK</t>
+  </si>
+  <si>
+    <t>Gold price below $5,000 as investors wait on Fed guidance for clues  Yahoo Finance UK</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxNMUUxWklvNENGNjNoaF9ER2hvVEp0ZjNEb3hWUHdqY0lzQW9VZWd3VGtRQ1VmcWMyT2wzOUh0X0pqbXNGLWduMGFlajhPZUlaTlpfREhfdXRWbDFUem1tRnlkRVNrSXUtaWhVRERwRUNlTTFHcVYxMFFwNWN0dzVwVXdja09wa0U1SmxlTFZYdWRZa01MdWJtOGI1R1J3RTdZSFdaOU51dkFRRVBrb181UnhQWUNhS2g3YjVfV1JKODNfWjJvQzlxVFVxMGRIZw?oc=5</t>
+  </si>
+  <si>
+    <t>ADMA Biologics to Report Fourth Quarter and Full Year 2025 Financial Results on February 25, 2026 - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>ADMA Biologics to Report Fourth Quarter and Full Year 2025 Financial Results on February 25, 2026  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOelJTNnhWN2JPN1hGaXYwX200Y1ZYcUJLdkh1bUpNUGk4NGVfSlZqWTl3eGwyWUd4QjBFeXYtTW5mQzliSnVtOUk3X0NObTZDTW1jMGl0SDk0VUtMWjFGdS1EVTlHdzN1Y1B5M1VDWEJEaTRCbkhpdFNFbkxsQ0JHWkNrVWUyQTN5Mnc?oc=5</t>
+  </si>
+  <si>
+    <t>Apple decouples from Nasdaq, offering alternative to AI-fueled volatility - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Apple decouples from Nasdaq, offering alternative to AI-fueled volatility  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQc3ZPY2hTcHBmTk1zRXI2czJhSnEwaDRONDl3SmhXbEVOZWdEd3FJdkNBVDc2Q0lPalVFY0FZbGNLNkRla1BoNHFybTF0ZGkydVNkTmRRbjNMMjkyYlhwTTJnVER3TjdzUTVsd3N2QWtCWDdDZ0xGNjNpQ0dnaVpRcThjRQ?oc=5</t>
+  </si>
+  <si>
+    <t>Kyndryl (KD) Soars 11% on Financial Statement Compliance - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Kyndryl (KD) Soars 11% on Financial Statement Compliance  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPS09EMmQ0Z3BLd3VyWVFYZU9PUG8wMkFnNkxnQUYwTE9tdHQ5dXM3djhDQkJQN3pOcGsyRHdNUFBoZFY2VmxLdWQ5Qm1tUjE0RHhnTjRjM2V1LUtDSGtWdkx1X2g4VHU1NXFpbTRxRTJjcUpFaXZOSVR4bElxTkNYaQ?oc=5</t>
+  </si>
+  <si>
+    <t>Luotea plc will publish Financial Statements Release for 2025 on 27 February 2026 - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Luotea plc will publish Financial Statements Release for 2025 on 27 February 2026  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOV2t0cklVS29jTS1qa1Z3eDhNQms4bWVLUmV3MW94QTVMZnFJVXltbENYZmlPdmRneDM2RWJZbkxtT2o1WU1kdUVNSklKLXJfWU5VMWhMRmJuTzhkaW1jSGtnaFpmREk5Y2liRWVJb1FULWVubEdmTEtQX1ZUSmxRcXdveWJtdWsxODZuc2NR?oc=5</t>
+  </si>
+  <si>
+    <t>Wingstop Inc. Reports Fourth Quarter and Fiscal Year 2025 Financial Results - PR Newswire</t>
+  </si>
+  <si>
+    <t>Wingstop Inc. Reports Fourth Quarter and Fiscal Year 2025 Financial Results  PR Newswire</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxObjkzcjdQNW03cmVjV01GdWxoV2VjT2pZWEN6amlMSWw0UUotbk42TEt6cDVXZmp5Mnd1aG9QUk9Zb2owOC1BYXZjTW53RmoyWlFqNzV1ZmhSOTd0dFNJXzF5YUJsempmSDEwbVRXRk9CWmVOaXVNNG1lX2E2R3FhTFhrZDE2eDdGZVhDWnJDY1NzdF96M2VyQUVaNjIxbkVDdGhabnB3TkZPT2RzNlVmRk1iTnhzTnhDSnM0QmpVbnM5YkZ0M19aOFZ3?oc=5</t>
   </si>
   <si>
     <t>‘He’s jumping in all the way’: A Trump financial regulator backs prediction markets in their clash against states - Politico</t>
@@ -2249,13 +2312,40 @@
     <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxNX3hNc0hjMW1FVW5WaVZOSnhIcmlMQjYxc1gycEdZWkczSXFPeUF0ZVh6SWg0RERvbVE1eXoyN2FyY0J0R2VQbmt0ZjZDY3BNRFpxMk5hZm4tNDl3eDdyM2tnSGFxN19udmV0LVlJbmpwbzI2cUh5WU5YZVdvYWVHRi04U2hlUnNVMm5tdE5n?oc=5</t>
   </si>
   <si>
-    <t>Gold price below $5,000 as investors wait on Fed guidance for clues - Yahoo Finance UK</t>
-  </si>
-  <si>
-    <t>Gold price below $5,000 as investors wait on Fed guidance for clues  Yahoo Finance UK</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxNMUUxWklvNENGNjNoaF9ER2hvVEp0ZjNEb3hWUHdqY0lzQW9VZWd3VGtRQ1VmcWMyT2wzOUh0X0pqbXNGLWduMGFlajhPZUlaTlpfREhfdXRWbDFUem1tRnlkRVNrSXUtaWhVRERwRUNlTTFHcVYxMFFwNWN0dzVwVXdja09wa0U1SmxlTFZYdWRZa01MdWJtOGI1R1J3RTdZSFdaOU51dkFRRVBrb181UnhQWUNhS2g3YjVfV1JKODNfWjJvQzlxVFVxMGRIZw?oc=5</t>
+    <t>MFA Financial, Inc. Announces Fourth Quarter and Full Year 2025 Financial Results - Yahoo Finance Singapore</t>
+  </si>
+  <si>
+    <t>MFA Financial, Inc. Announces Fourth Quarter and Full Year 2025 Financial Results  Yahoo Finance Singapore</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPWXRuWEJ5bFhBN1VnUngzblhLVDkzMDJkaTFWSmI4NnhzSkh1NTZpX2FWeEJIM0lNLURPU3o3bU1Uc3BpLU9CeW1Sek5OSDRPYnhNY3l6bDJNdEpsdXk3UjFLVU85OGZsVVkxeFN4QjdPQXVDdHlES0tteDZ3eS1aM1dTRnp5Y3FhdHRN?oc=5</t>
+  </si>
+  <si>
+    <t>Will Chen joins Westfield Specialty as U.S. Chief Financial Officer - PR Newswire</t>
+  </si>
+  <si>
+    <t>Will Chen joins Westfield Specialty as U.S. Chief Financial Officer  PR Newswire</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVVpzWURrVFNsVXlfeHJ5VlE0MWpPNHJnYV9FRFhyR1lzU29iOWRmTURzUW4yVDlGUFFndUl4VzBKSGlxOWV1bVlIS1BCTmlscy1OQzk2Y1FUNnhEN2ZjV2JORmtKOWZvaDdxeGhZdGxGVlVaQThlSjBBYXJfeS10VkNMMXVQaTllMGh4V0VJc0JaVVRURHZSTWVrenJyRkJXUHc0TWk4ZzR0V3R4UFpfVldfNEppUEhrX2ZVTUl3?oc=5</t>
+  </si>
+  <si>
+    <t>FOX23 Investigates: Tulsa families question credit union they used to finance pools - fox23.com</t>
+  </si>
+  <si>
+    <t>FOX23 Investigates: Tulsa families question credit union they used to finance pools  fox23.com</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxOSXF3Qlc4SzVaLUtQS1lRT0RGS3BQVUN2aEtPQjVBcThGV2c2M2gzaTBSVFVTOUhkb0VGSlF2d3JMenA2eGdmU1FQODI1NlB6Y2ZKckV3ZTY4LWx3NnlnYlFFLUNlTzdfWXpCLUs0QjZjWG9PUmxQWE9XLTNmYlZ4VDBtLTREWFMyWkpLazlDN1J1aEJCX25qYU9OSUlkSzBaaTBrQXJTU3JQRk1JZHJOX2k2TnJyN0ZMdkJPQ29meUFJOVBDQ3FhY2lULWpOR3ROTml5VW5Ma0ZYZnR3LTNkdkNhY1FNbWxtdlZJX2hZaWE?oc=5</t>
+  </si>
+  <si>
+    <t>Scottish Water taps Oracle to support agile transformation - Oracle</t>
+  </si>
+  <si>
+    <t>Scottish Water taps Oracle to support agile transformation  Oracle</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE04cnh1aG1Vcnp6bzI0R2ozajBGckJLcy10RG9JdTFlbDVacWRXSzA2V0hZa3d3bHVNY1NiVGRNVDNIM0pHVVM4SEozUG5zOFRmTmU3NVl4X2FyVDVq?oc=5</t>
   </si>
   <si>
     <t>OFS Financial Services Provides Insurance So You Don’t Have to Choose Between Care and Cost - ThurstonTalk</t>
@@ -2267,40 +2357,94 @@
     <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNcEdHdTZEVDAxNFQyT3pxNGhSdlpSU2FkdG5FYVZEY2lNU1R4YWRzV2lfalhzS005OUdDNzlpd1VuSkZhN3hTMGVqNTdZMVF6a1NRNU9lWjlLYlZaNklGTWcwVDVrYllxTFRVbXF3Umk3dzBoNkpLVlVnWjRQMXgxbThDZkZYb1puRDROU0tldHlaeXduV05qaUxBS240SGZ5UVdQbDlCZ0x4bUQxQ0NrVVJRTnZNVi1TcWE4eFJtZU9SSUVoc1haakg0Zw?oc=5</t>
   </si>
   <si>
-    <t>ADMA Biologics to Report Fourth Quarter and Full Year 2025 Financial Results on February 25, 2026 - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>ADMA Biologics to Report Fourth Quarter and Full Year 2025 Financial Results on February 25, 2026  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOelJTNnhWN2JPN1hGaXYwX200Y1ZYcUJLdkh1bUpNUGk4NGVfSlZqWTl3eGwyWUd4QjBFeXYtTW5mQzliSnVtOUk3X0NObTZDTW1jMGl0SDk0VUtMWjFGdS1EVTlHdzN1Y1B5M1VDWEJEaTRCbkhpdFNFbkxsQ0JHWkNrVWUyQTN5Mnc?oc=5</t>
-  </si>
-  <si>
-    <t>Apple decouples from Nasdaq, offering alternative to AI-fueled volatility - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Apple decouples from Nasdaq, offering alternative to AI-fueled volatility  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQc3ZPY2hTcHBmTk1zRXI2czJhSnEwaDRONDl3SmhXbEVOZWdEd3FJdkNBVDc2Q0lPalVFY0FZbGNLNkRla1BoNHFybTF0ZGkydVNkTmRRbjNMMjkyYlhwTTJnVER3TjdzUTVsd3N2QWtCWDdDZ0xGNjNpQ0dnaVpRcThjRQ?oc=5</t>
-  </si>
-  <si>
-    <t>Kyndryl (KD) Soars 11% on Financial Statement Compliance - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Kyndryl (KD) Soars 11% on Financial Statement Compliance  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPS09EMmQ0Z3BLd3VyWVFYZU9PUG8wMkFnNkxnQUYwTE9tdHQ5dXM3djhDQkJQN3pOcGsyRHdNUFBoZFY2VmxLdWQ5Qm1tUjE0RHhnTjRjM2V1LUtDSGtWdkx1X2g4VHU1NXFpbTRxRTJjcUpFaXZOSVR4bElxTkNYaQ?oc=5</t>
-  </si>
-  <si>
-    <t>Video: FOX23 Investigates: Tulsa families question credit union they used to finance pools - fox23.com</t>
-  </si>
-  <si>
-    <t>Video: FOX23 Investigates: Tulsa families question credit union they used to finance pools  fox23.com</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxNYlB5bmZWdHFBeVJWWGhxNmY5bmRZU1Azd25LNnZHLWpYVkwxWmlnTDF2QXlKb2JZcEJlbGVTT1lScHkxeU1od1N4TVotZkJvT3lRYV9sejB2QXNvWDRhTzljZTVjV2g4NUdTenN0LWpHdHhZQjBxRlRBOFpkSzBKZmVYVHhXS1RHZWRyM1FJa01UVDhqZXh5VVV5dUJPMUNVdHluRXlUN2Nyby1CalB3NkFMYW1UZ1Z5b2F2NkVtVVV3UGFjU2FwdTVjdjhzU0Z0N2hjb0Q1Z09YUmFYN0d2ZmJONFlVYzlOclMzYnhwWDZURWRHUUE?oc=5</t>
+    <t>Nvidia in focus: Meta partnership expanded, Arm stake sold - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Nvidia in focus: Meta partnership expanded, Arm stake sold  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOSFdMSEFMSDJ5Mk1nTk5xdkhTTHdDQzlJS3NZY2xKTnloYy1Nb2FQYk9QdHBoR3hqZlNOQkxzVHFTbEI5NGJ2OFA0Ulc2clhVR09nYTc3OU5jdVhMTFRDV0w2dERzWVVVQmJJWURFWUh3OEh0OTYwM2lHMkN2em9qcXotNE1sa1dzZjNaU1pn?oc=5</t>
+  </si>
+  <si>
+    <t>Verastem Oncology to Report Fourth Quarter and Full Year 2025 Financial Results on March 4, 2026 - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Verastem Oncology to Report Fourth Quarter and Full Year 2025 Financial Results on March 4, 2026  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOeHVlU1QyOWNaQnd4MlQ3dkF0RXdPczhfc0NJRDZpd2c1bDNQQThrblhraWQ2S0xhdk1kVGtDTkRrVktTZFE4c0hkcGlYS1hRdVYya0JnUlNrcEFQY09tcHBSNlhQS2pkdVByS3pFc0gydl9NOGRoQW5zX2ZLT0NZMzNkem9pRjBtQnhTZ3lB?oc=5</t>
+  </si>
+  <si>
+    <t>Charleston launches Financial Empowerment Center for residents - Live 5 News</t>
+  </si>
+  <si>
+    <t>Charleston launches Financial Empowerment Center for residents  Live 5 News</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOQXhWZFN3ek1UV3F2UjBhVXhKZlpva3pXUFRBdnJtYk5LYUc0aHdYLVlTbEw2MDRyd3hjZlNSdmUtVHEzb0FPT1RQRWtMbWN4LXdzS3c0bWZ1bEU5UDJ1V2J0OFJGemNmSEg5RE5zandQTXJPYjNIUzVucGdIcVBORTFPdldCY3Q1SjMtQjA2NS1BMmdoTkM0RXhwdXbSAbABQVVfeXFMTVFLTldMZmRxZnBLS3ltT2JQaDJFcEJWR2tMZXlVOWtNSWxDbVRMNDJUSlk1WkJVYndMSmMxTlNkT3VpclJtak1DcGtKSDR5eTIzeGtGWk9hVzBtOEZUcndOeDFtQXJLbGgxRl9mWTRzQVpydC1MX2RXZVc5VWN6cDQyc1RqRnVkeklSRUV1SU9tcHZheFRHbTFkcTFjQkI1OW9FdTF6LV9lT3FNSXNKWjY?oc=5</t>
+  </si>
+  <si>
+    <t>Palantir upgraded, Workday downgraded: Wall Street's top analyst calls - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Palantir upgraded, Workday downgraded: Wall Street's top analyst calls  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPQXBvZnBsVHRXNUF0NWpMRkFBbFJHeV9kQmFXMUxDbTRPcmszOW1TRmVDQXVROEpiLUpmQURXS2x0cnRncWZLYTRiYktrNW5PNGhfdXJrU1J5SEMzZHRMdEJ6TmxGOWt5eXRIelcyR3pPY2M2XzdrbldtazhyVGhxWXdxem9Ecm45VDVTT29kdTE?oc=5</t>
+  </si>
+  <si>
+    <t>Brian Armstrong Reveals Retail Users 'Buying The Dip' In Bitcoin, Ethereum: Coinbase CEO Says, 'They Have Diamond Hands' - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Brian Armstrong Reveals Retail Users 'Buying The Dip' In Bitcoin, Ethereum: Coinbase CEO Says, 'They Have Diamond Hands'  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPRGRKMXhSa2ZDZGZVbXRVZGpiYXNrOHpWc2FxWVpnSUMwVmtObExFdTlrSktGd0p1WlZaX1g4b3JacW9rRnVtMnpPM0tpSFIxRmJGS1cyX2ljLV9zLWxHc05qeXc3UUNBOU9PSDY4aTFMT040b3REODFGem9ULXM5SWtrSDROTzdZd0E?oc=5</t>
+  </si>
+  <si>
+    <t>Ericsson and Mastercard enhance global digital money movement and accelerate digital financial inclusion - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Ericsson and Mastercard enhance global digital money movement and accelerate digital financial inclusion  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNWk9Ha2ZHM3NrNmNMMjh2ZFlaX0dxdXdiYnBucXpHNTZZcTE1RGl6SGRCUzdMSW9yYzNqTGxRckhYT0NwUzhHVkxYSGcydVlrbTl6NzdyeG9SOW1aRmpUZ041T1V2OVNRdmRlaHVQVHRsWGpPUUlIc3I1a2dwWWJoTDFIQU90TmhxR2NQanZ1YmNkZw?oc=5</t>
+  </si>
+  <si>
+    <t>Swift Current Energy Secures Project Financing and Tax Equity for 122 MW Energy Facility in Maine - PR Newswire</t>
+  </si>
+  <si>
+    <t>Swift Current Energy Secures Project Financing and Tax Equity for 122 MW Energy Facility in Maine  PR Newswire</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxOa2ZNV3VUc3ZrNktDSF9Hc1BaeGh4aFJaQWg1Uk5oSDFsdy1qQkRKSDVtWjVUV3pnVzloNHFWZ1BnUld1UGJpcnJLLUJsV2V2SVJMcW9QX0RXNDVvLXVhcUpiLXVWSWU0bWdsa3k4SnQ5OXFJeFFwQS13Wk00eGQ1RFc4WkxBcGk0azBXc1hYT3NFenk4R1hHYmFqTDZicXJvdVpiYWtXUFVjT3VBenZuMkx1UFJqSDhIVFczVUlTdl94QmVVWGJsSXd1TTRSWUx5NmVvR2ZxelBSOEtFNkZEU1laNzdOUDY3?oc=5</t>
+  </si>
+  <si>
+    <t>Harrow To Report Fourth Quarter and Year-End 2025 Financial Results After Market Close on March 2, 2026 - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Harrow To Report Fourth Quarter and Year-End 2025 Financial Results After Market Close on March 2, 2026  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOVVB3alBRUWdJS0kxb3BYclo1VS1PclRzLVUwTmluRFFQX1JnZUVNUVEwR1JvcW94cWhnYWtuSTZ5QlA4TjBMTXNyUm0wZUt3YzhGdFpYbDBiQjBEaUpmVkFjZFNiYXY2bUZaOXJlelFaZzdSVjRmS3lsN2JEbmtxT2JJV2s?oc=5</t>
+  </si>
+  <si>
+    <t>Meta CEO Mark Zuckerberg set to testify in teen social media addiction suit - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Meta CEO Mark Zuckerberg set to testify in teen social media addiction suit  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOTDJaZUVoeXJuVjBuTUNrMU5GbEhncFgwVTZ5X0Q3bGFXNEhYakxDM3Q1VnQ1eS1rMzRDcERUSWZKX2xRcTVPNjFXbWJNTHV6SXVlcTBZd0tpTlZ2ZlZVb3JIMjZaSm1iM0UwR3h3LXdkU09MM2tmNDVFOXZmQldqQVkzV1hFRTFaSG1mQXF0OGNMY3hQbXZZa2dodjZJbkhVc1RwU0IwdGtIN2FuaURjeG11bGYxcVo5eHFsZXdn?oc=5</t>
+  </si>
+  <si>
+    <t>Recursion to Report Fourth Quarter and Full Year 2025 Business Updates and Financial Results on February 25 - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>Recursion to Report Fourth Quarter and Full Year 2025 Business Updates and Financial Results on February 25  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNUktiOHpfaDBaekR6MmlpQVVTOXZ6TUZKYWxzblF4eE1acE54eXlNYWwtOVdYbmxadjhKNk5Vc1ZXVFFlNzQ1Zkt1Y0hfbDBlQ2VPOEM1Q3lEQ0FNam9SWkh2ZWFmZXE0azdWalotcFZmVzJTWGhVdWp3ZlJWRnk0VUlTRFFQNGtaRWc?oc=5</t>
   </si>
   <si>
     <t>Hawaiʻi Was Once A National Leader In Long-Term Care Financing - Honolulu Civil Beat</t>
@@ -2312,15 +2456,6 @@
     <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQNkJBUVJVMUd1Mld5MlFVSkZVYXNnUFV1MF9EeEVKX1dSSWxpcGpUbjBGR1BTdTBEem05UmlYdW1HdXlISHhhakVjYndQQUpRU3QxY1R0MFdiSFpNd0xOdE9La0Z2NFlUUkZhUWxHMC1SQ1gzZ1BDYXVVN1NZUElid0dLdmUwMVRyay04VmpnR2dkTVU4M1QtcU5PSlhyaF9kV1hyQQ?oc=5</t>
   </si>
   <si>
-    <t>Scottish Water taps Oracle to support agile transformation - Oracle</t>
-  </si>
-  <si>
-    <t>Scottish Water taps Oracle to support agile transformation  Oracle</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE04cnh1aG1Vcnp6bzI0R2ozajBGckJLcy10RG9JdTFlbDVacWRXSzA2V0hZa3d3bHVNY1NiVGRNVDNIM0pHVVM4SEozUG5zOFRmTmU3NVl4X2FyVDVq?oc=5</t>
-  </si>
-  <si>
     <t>The adoption and efficacy of large language models in US consumer financial complaints - Nature</t>
   </si>
   <si>
@@ -2339,139 +2474,13 @@
     <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9YZXY5aVdtbFpHdk1mQVZvaDgtWEdyaHpYd3N0a0dWZ3NQYlpfaEtwY3c1c2ZDQ0lfX05jdzBGaGZZZGR2UjhiZnZHMFJVa1FmVDFDSVIzbTBCMl9SNG9JVVMwTHl2MnVheEFfbXFWamQ?oc=5</t>
   </si>
   <si>
-    <t>Luotea plc will publish Financial Statements Release for 2025 on 27 February 2026 - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Luotea plc will publish Financial Statements Release for 2025 on 27 February 2026  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOV2t0cklVS29jTS1qa1Z3eDhNQms4bWVLUmV3MW94QTVMZnFJVXltbENYZmlPdmRneDM2RWJZbkxtT2o1WU1kdUVNSklKLXJfWU5VMWhMRmJuTzhkaW1jSGtnaFpmREk5Y2liRWVJb1FULWVubEdmTEtQX1ZUSmxRcXdveWJtdWsxODZuc2NR?oc=5</t>
-  </si>
-  <si>
-    <t>Swift Current Energy Secures Project Financing and Tax Equity for 122 MW Energy Facility in Maine - PR Newswire</t>
-  </si>
-  <si>
-    <t>Swift Current Energy Secures Project Financing and Tax Equity for 122 MW Energy Facility in Maine  PR Newswire</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxOa2ZNV3VUc3ZrNktDSF9Hc1BaeGh4aFJaQWg1Uk5oSDFsdy1qQkRKSDVtWjVUV3pnVzloNHFWZ1BnUld1UGJpcnJLLUJsV2V2SVJMcW9QX0RXNDVvLXVhcUpiLXVWSWU0bWdsa3k4SnQ5OXFJeFFwQS13Wk00eGQ1RFc4WkxBcGk0azBXc1hYT3NFenk4R1hHYmFqTDZicXJvdVpiYWtXUFVjT3VBenZuMkx1UFJqSDhIVFczVUlTdl94QmVVWGJsSXd1TTRSWUx5NmVvR2ZxelBSOEtFNkZEU1laNzdOUDY3?oc=5</t>
-  </si>
-  <si>
-    <t>Wingstop Inc. Reports Fourth Quarter and Fiscal Year 2025 Financial Results - PR Newswire</t>
-  </si>
-  <si>
-    <t>Wingstop Inc. Reports Fourth Quarter and Fiscal Year 2025 Financial Results  PR Newswire</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxObjkzcjdQNW03cmVjV01GdWxoV2VjT2pZWEN6amlMSWw0UUotbk42TEt6cDVXZmp5Mnd1aG9QUk9Zb2owOC1BYXZjTW53RmoyWlFqNzV1ZmhSOTd0dFNJXzF5YUJsempmSDEwbVRXRk9CWmVOaXVNNG1lX2E2R3FhTFhrZDE2eDdGZVhDWnJDY1NzdF96M2VyQUVaNjIxbkVDdGhabnB3TkZPT2RzNlVmRk1iTnhzTnhDSnM0QmpVbnM5YkZ0M19aOFZ3?oc=5</t>
-  </si>
-  <si>
-    <t>MFA Financial, Inc. Announces Fourth Quarter and Full Year 2025 Financial Results - Yahoo Finance Singapore</t>
-  </si>
-  <si>
-    <t>MFA Financial, Inc. Announces Fourth Quarter and Full Year 2025 Financial Results  Yahoo Finance Singapore</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPWXRuWEJ5bFhBN1VnUngzblhLVDkzMDJkaTFWSmI4NnhzSkh1NTZpX2FWeEJIM0lNLURPU3o3bU1Uc3BpLU9CeW1Sek5OSDRPYnhNY3l6bDJNdEpsdXk3UjFLVU85OGZsVVkxeFN4QjdPQXVDdHlES0tteDZ3eS1aM1dTRnp5Y3FhdHRN?oc=5</t>
-  </si>
-  <si>
-    <t>Will Chen joins Westfield Specialty as U.S. Chief Financial Officer - PR Newswire</t>
-  </si>
-  <si>
-    <t>Will Chen joins Westfield Specialty as U.S. Chief Financial Officer  PR Newswire</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPVVpzWURrVFNsVXlfeHJ5VlE0MWpPNHJnYV9FRFhyR1lzU29iOWRmTURzUW4yVDlGUFFndUl4VzBKSGlxOWV1bVlIS1BCTmlscy1OQzk2Y1FUNnhEN2ZjV2JORmtKOWZvaDdxeGhZdGxGVlVaQThlSjBBYXJfeS10VkNMMXVQaTllMGh4V0VJc0JaVVRURHZSTWVrenJyRkJXUHc0TWk4ZzR0V3R4UFpfVldfNEppUEhrX2ZVTUl3?oc=5</t>
-  </si>
-  <si>
-    <t>FOX23 Investigates: Tulsa families question credit union they used to finance pools - fox23.com</t>
-  </si>
-  <si>
-    <t>FOX23 Investigates: Tulsa families question credit union they used to finance pools  fox23.com</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxOSXF3Qlc4SzVaLUtQS1lRT0RGS3BQVUN2aEtPQjVBcThGV2c2M2gzaTBSVFVTOUhkb0VGSlF2d3JMenA2eGdmU1FQODI1NlB6Y2ZKckV3ZTY4LWx3NnlnYlFFLUNlTzdfWXpCLUs0QjZjWG9PUmxQWE9XLTNmYlZ4VDBtLTREWFMyWkpLazlDN1J1aEJCX25qYU9OSUlkSzBaaTBrQXJTU3JQRk1JZHJOX2k2TnJyN0ZMdkJPQ29meUFJOVBDQ3FhY2lULWpOR3ROTml5VW5Ma0ZYZnR3LTNkdkNhY1FNbWxtdlZJX2hZaWE?oc=5</t>
-  </si>
-  <si>
-    <t>SME finance: the geographic gap in equity financing - Centre for Cities</t>
-  </si>
-  <si>
-    <t>SME finance: the geographic gap in equity financing  Centre for Cities</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQMnB0NmlfT2UxUFBXcTN3Um9NOU03UzVYNTdwNmMweC0tbVVDVk1hWVEyQ2hjUVhfblpfY0doUGhpckdHMm9vUDJPXzI3LVpQNG1aR09PbUlpeGVMTzBCTi1QYmhvRjJyR1hiUlBMcWFWVjVpZER2SkxiSUhKeXVrQU5TeEFxY1VIMmF5SjBRWGdLb3c?oc=5</t>
-  </si>
-  <si>
-    <t>Nvidia in focus: Meta partnership expanded, Arm stake sold - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Nvidia in focus: Meta partnership expanded, Arm stake sold  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOSFdMSEFMSDJ5Mk1nTk5xdkhTTHdDQzlJS3NZY2xKTnloYy1Nb2FQYk9QdHBoR3hqZlNOQkxzVHFTbEI5NGJ2OFA0Ulc2clhVR09nYTc3OU5jdVhMTFRDV0w2dERzWVVVQmJJWURFWUh3OEh0OTYwM2lHMkN2em9qcXotNE1sa1dzZjNaU1pn?oc=5</t>
-  </si>
-  <si>
-    <t>Verastem Oncology to Report Fourth Quarter and Full Year 2025 Financial Results on March 4, 2026 - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Verastem Oncology to Report Fourth Quarter and Full Year 2025 Financial Results on March 4, 2026  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOeHVlU1QyOWNaQnd4MlQ3dkF0RXdPczhfc0NJRDZpd2c1bDNQQThrblhraWQ2S0xhdk1kVGtDTkRrVktTZFE4c0hkcGlYS1hRdVYya0JnUlNrcEFQY09tcHBSNlhQS2pkdVByS3pFc0gydl9NOGRoQW5zX2ZLT0NZMzNkem9pRjBtQnhTZ3lB?oc=5</t>
-  </si>
-  <si>
-    <t>Palantir upgraded, Workday downgraded: Wall Street's top analyst calls - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Palantir upgraded, Workday downgraded: Wall Street's top analyst calls  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPQXBvZnBsVHRXNUF0NWpMRkFBbFJHeV9kQmFXMUxDbTRPcmszOW1TRmVDQXVROEpiLUpmQURXS2x0cnRncWZLYTRiYktrNW5PNGhfdXJrU1J5SEMzZHRMdEJ6TmxGOWt5eXRIelcyR3pPY2M2XzdrbldtazhyVGhxWXdxem9Ecm45VDVTT29kdTE?oc=5</t>
-  </si>
-  <si>
-    <t>Brian Armstrong Reveals Retail Users 'Buying The Dip' In Bitcoin, Ethereum: Coinbase CEO Says, 'They Have Diamond Hands' - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Brian Armstrong Reveals Retail Users 'Buying The Dip' In Bitcoin, Ethereum: Coinbase CEO Says, 'They Have Diamond Hands'  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPRGRKMXhSa2ZDZGZVbXRVZGpiYXNrOHpWc2FxWVpnSUMwVmtObExFdTlrSktGd0p1WlZaX1g4b3JacW9rRnVtMnpPM0tpSFIxRmJGS1cyX2ljLV9zLWxHc05qeXc3UUNBOU9PSDY4aTFMT040b3REODFGem9ULXM5SWtrSDROTzdZd0E?oc=5</t>
-  </si>
-  <si>
-    <t>Ericsson and Mastercard enhance global digital money movement and accelerate digital financial inclusion - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Ericsson and Mastercard enhance global digital money movement and accelerate digital financial inclusion  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNWk9Ha2ZHM3NrNmNMMjh2ZFlaX0dxdXdiYnBucXpHNTZZcTE1RGl6SGRCUzdMSW9yYzNqTGxRckhYT0NwUzhHVkxYSGcydVlrbTl6NzdyeG9SOW1aRmpUZ041T1V2OVNRdmRlaHVQVHRsWGpPUUlIc3I1a2dwWWJoTDFIQU90TmhxR2NQanZ1YmNkZw?oc=5</t>
-  </si>
-  <si>
-    <t>Harrow To Report Fourth Quarter and Year-End 2025 Financial Results After Market Close on March 2, 2026 - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Harrow To Report Fourth Quarter and Year-End 2025 Financial Results After Market Close on March 2, 2026  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOVVB3alBRUWdJS0kxb3BYclo1VS1PclRzLVUwTmluRFFQX1JnZUVNUVEwR1JvcW94cWhnYWtuSTZ5QlA4TjBMTXNyUm0wZUt3YzhGdFpYbDBiQjBEaUpmVkFjZFNiYXY2bUZaOXJlelFaZzdSVjRmS3lsN2JEbmtxT2JJV2s?oc=5</t>
-  </si>
-  <si>
-    <t>Meta CEO Mark Zuckerberg set to testify in teen social media addiction suit - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Meta CEO Mark Zuckerberg set to testify in teen social media addiction suit  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOTDJaZUVoeXJuVjBuTUNrMU5GbEhncFgwVTZ5X0Q3bGFXNEhYakxDM3Q1VnQ1eS1rMzRDcERUSWZKX2xRcTVPNjFXbWJNTHV6SXVlcTBZd0tpTlZ2ZlZVb3JIMjZaSm1iM0UwR3h3LXdkU09MM2tmNDVFOXZmQldqQVkzV1hFRTFaSG1mQXF0OGNMY3hQbXZZa2dodjZJbkhVc1RwU0IwdGtIN2FuaURjeG11bGYxcVo5eHFsZXdn?oc=5</t>
-  </si>
-  <si>
-    <t>Recursion to Report Fourth Quarter and Full Year 2025 Business Updates and Financial Results on February 25 - Yahoo Finance</t>
-  </si>
-  <si>
-    <t>Recursion to Report Fourth Quarter and Full Year 2025 Business Updates and Financial Results on February 25  Yahoo Finance</t>
-  </si>
-  <si>
-    <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNUktiOHpfaDBaekR6MmlpQVVTOXZ6TUZKYWxzblF4eE1acE54eXlNYWwtOVdYbmxadjhKNk5Vc1ZXVFFlNzQ1Zkt1Y0hfbDBlQ2VPOEM1Q3lEQ0FNam9SWkh2ZWFmZXE0azdWalotcFZmVzJTWGhVdWp3ZlJWRnk0VUlTRFFQNGtaRWc?oc=5</t>
+    <t>NewAmsterdam Pharma Reports Full Year 2025 Financial Results and Provides Corporate Update - Yahoo Finance</t>
+  </si>
+  <si>
+    <t>NewAmsterdam Pharma Reports Full Year 2025 Financial Results and Provides Corporate Update  Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxPM0xkQ2h2UEN6cXdCRUprYkdxM3dSWV9mbG40R0tLcGtxY1BUaUJaU3hTaDM5dlcwRDVwcVU2eFZEbnczRnliY2ZncmxGbzNMa3lxSUM2dklkeW5Tc19GS2F1TnI2UTVVbkRsNlhndi1VWG5hX2tFOTBnYk9KNjdJa1lTbXJaQW82dUVz?oc=5</t>
   </si>
   <si>
     <t>Mortgage Rates Today, Wednesday, February 18: Rates Remain Low</t>
@@ -2573,6 +2582,15 @@
     <t>https://stockmarketwatch.com/stock-market-news/exxonmobil-expands-guyana-gas-strategy-jj-commits-1-billion-to-pennsylvania-expansion/58720/</t>
   </si>
   <si>
+    <t>Why Nvidia’s deal with Meta is an ‘Intel killer,’ according to this analyst</t>
+  </si>
+  <si>
+    <t>The use of Nvidia CPUs could signal a significant shift toward Arm-based chips in the data center.</t>
+  </si>
+  <si>
+    <t>https://www.marketwatch.com/story/why-nvidias-deal-with-meta-is-an-intel-killer-according-to-this-analyst-a531f80d?mod=mw_rss_topstories</t>
+  </si>
+  <si>
     <t>How Amazon’s ‘underappreciated’ AI potential could drive the stock 50% higher</t>
   </si>
   <si>
@@ -2654,13 +2672,22 @@
     <t>https://www.marketwatch.com/story/moderna-got-the-fda-to-change-its-mind-and-review-its-flu-vaccine-after-some-concessions-04c3f38e?mod=mw_rss_topstories</t>
   </si>
   <si>
-    <t>Why a 40-year Wall Street veteran is telling clients to sell everything American</t>
-  </si>
-  <si>
-    <t>Andy Constan says the rest of the world now offers more opportunities.</t>
-  </si>
-  <si>
-    <t>https://www.marketwatch.com/story/why-a-40-year-wall-street-veteran-is-telling-clients-to-sell-everything-american-77e50ae5?mod=mw_rss_topstories</t>
+    <t>Laureate Education Q4 2025 Earnings Preview</t>
+  </si>
+  <si>
+    <t>https://seekingalpha.com/news/4553468-laureate-education-q4-2025-earnings-preview?utm_source=feed_news_all&amp;utm_medium=referral&amp;feed_item_type=news</t>
+  </si>
+  <si>
+    <t>Sprott Q4 2025 Earnings Preview</t>
+  </si>
+  <si>
+    <t>https://seekingalpha.com/news/4553467-sprott-q4-2025-earnings-preview?utm_source=feed_news_all&amp;utm_medium=referral&amp;feed_item_type=news</t>
+  </si>
+  <si>
+    <t>Talkspace Q4 2025 Earnings Preview</t>
+  </si>
+  <si>
+    <t>https://seekingalpha.com/news/4553466-talkspace-q4-2025-earnings-preview?utm_source=feed_news_all&amp;utm_medium=referral&amp;feed_item_type=news</t>
   </si>
   <si>
     <t>ICON rises as Cowen upgrades after recent selloff</t>
@@ -2687,24 +2714,6 @@
     <t>https://seekingalpha.com/news/4553453-quad-projects-net-sales-decline-of-1-percent-to-5-percent-in-2026-as-targeted-print-and?utm_source=feed_news_all&amp;utm_medium=referral&amp;feed_item_type=news</t>
   </si>
   <si>
-    <t>Most and least shorted energy stocks with over $2B market cap as of mid-Feb</t>
-  </si>
-  <si>
-    <t>https://seekingalpha.com/news/4553446-most-and-least-shorted-large-cap-energy-stocks-as-of-mid-feb?utm_source=feed_news_all&amp;utm_medium=referral&amp;feed_item_type=news</t>
-  </si>
-  <si>
-    <t>Pediatrix Medical Group Q4 2025 Earnings Preview</t>
-  </si>
-  <si>
-    <t>https://seekingalpha.com/news/4553445-pediatrix-medical-group-q4-2025-earnings-preview?utm_source=feed_news_all&amp;utm_medium=referral&amp;feed_item_type=news</t>
-  </si>
-  <si>
-    <t>Visteon Q4 2025 Earnings Preview</t>
-  </si>
-  <si>
-    <t>https://seekingalpha.com/news/4553444-visteon-q4-2025-earnings-preview?utm_source=feed_news_all&amp;utm_medium=referral&amp;feed_item_type=news</t>
-  </si>
-  <si>
     <t>SharonAI debuts on Nasdaq slightly above IPO price</t>
   </si>
   <si>
@@ -2765,12 +2774,6 @@
     <t>https://www.investing.com/news/stock-market-news/moodys-forecasts-upbeat-2026-profit-on-strong-demand-for-credit-ratings-4510892</t>
   </si>
   <si>
-    <t>LIVE: White House briefing with Karoline Leavitt</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=f0LW2vYWuag</t>
-  </si>
-  <si>
     <t>LIVE: House's Hakeem Jeffries holds a briefing in Washington</t>
   </si>
   <si>
@@ -2853,6 +2856,12 @@
   </si>
   <si>
     <t>https://www.youtube.com/watch?v=osMjcYVxqEg</t>
+  </si>
+  <si>
+    <t>BAE Systems sees years of growth in ‘new era’ of defense spending</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=eBgrSqQEDX4</t>
   </si>
   <si>
     <t>Candidaturas de empresas a linha de crédito à tesouraria devido ao mau tempo somam 905 milhões</t>
@@ -4039,7 +4048,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D431"/>
+  <dimension ref="A1:D432"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -8098,8 +8107,11 @@
       <c r="A290" t="s">
         <v>864</v>
       </c>
+      <c r="B290" t="s">
+        <v>865</v>
+      </c>
       <c r="C290" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="D290" t="s">
         <v>7</v>
@@ -8107,10 +8119,10 @@
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="C291" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="D291" t="s">
         <v>7</v>
@@ -8118,10 +8130,10 @@
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="C292" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="D292" t="s">
         <v>7</v>
@@ -8129,10 +8141,10 @@
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="C293" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="D293" t="s">
         <v>7</v>
@@ -8140,10 +8152,10 @@
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C294" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="D294" t="s">
         <v>7</v>
@@ -8151,10 +8163,10 @@
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="C295" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="D295" t="s">
         <v>7</v>
@@ -8162,10 +8174,10 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="C296" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="D296" t="s">
         <v>7</v>
@@ -8173,10 +8185,10 @@
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="C297" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="D297" t="s">
         <v>7</v>
@@ -8184,10 +8196,10 @@
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="C298" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="D298" t="s">
         <v>7</v>
@@ -8195,10 +8207,10 @@
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="C299" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="D299" t="s">
         <v>7</v>
@@ -8206,10 +8218,10 @@
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="C300" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="D300" t="s">
         <v>7</v>
@@ -8217,10 +8229,10 @@
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="C301" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="D301" t="s">
         <v>7</v>
@@ -8228,10 +8240,10 @@
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="C302" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="D302" t="s">
         <v>7</v>
@@ -8239,10 +8251,10 @@
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="C303" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="D303" t="s">
         <v>7</v>
@@ -8250,10 +8262,10 @@
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="C304" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="D304" t="s">
         <v>7</v>
@@ -8261,10 +8273,10 @@
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="C305" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="D305" t="s">
         <v>7</v>
@@ -8272,10 +8284,10 @@
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="C306" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="D306" t="s">
         <v>7</v>
@@ -8283,10 +8295,10 @@
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="C307" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="D307" t="s">
         <v>7</v>
@@ -8294,10 +8306,10 @@
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="C308" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="D308" t="s">
         <v>7</v>
@@ -8305,10 +8317,10 @@
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="C309" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="D309" t="s">
         <v>7</v>
@@ -8316,10 +8328,10 @@
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="C310" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="D310" t="s">
         <v>7</v>
@@ -8327,10 +8339,10 @@
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="C311" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="D311" t="s">
         <v>7</v>
@@ -8338,10 +8350,10 @@
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="C312" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="D312" t="s">
         <v>7</v>
@@ -8349,10 +8361,10 @@
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="C313" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="D313" t="s">
         <v>7</v>
@@ -8360,10 +8372,10 @@
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="C314" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="D314" t="s">
         <v>7</v>
@@ -8371,10 +8383,10 @@
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="C315" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="D315" t="s">
         <v>7</v>
@@ -8382,10 +8394,10 @@
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="C316" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="D316" t="s">
         <v>7</v>
@@ -8393,10 +8405,10 @@
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="C317" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="D317" t="s">
         <v>7</v>
@@ -8404,10 +8416,10 @@
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="C318" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="D318" t="s">
         <v>7</v>
@@ -8415,10 +8427,10 @@
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="C319" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="D319" t="s">
         <v>7</v>
@@ -8426,10 +8438,10 @@
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="C320" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="D320" t="s">
         <v>7</v>
@@ -8437,10 +8449,10 @@
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="C321" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="D321" t="s">
         <v>7</v>
@@ -8448,9 +8460,6 @@
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>928</v>
-      </c>
-      <c r="B322" t="s">
         <v>929</v>
       </c>
       <c r="C322" t="s">
@@ -8590,8 +8599,11 @@
       <c r="A332" t="s">
         <v>958</v>
       </c>
+      <c r="B332" t="s">
+        <v>959</v>
+      </c>
       <c r="C332" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="D332" t="s">
         <v>7</v>
@@ -8599,10 +8611,10 @@
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="C333" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="D333" t="s">
         <v>7</v>
@@ -8610,10 +8622,10 @@
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="C334" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="D334" t="s">
         <v>7</v>
@@ -8621,10 +8633,10 @@
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="C335" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="D335" t="s">
         <v>7</v>
@@ -8632,10 +8644,10 @@
     </row>
     <row r="336" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="C336" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="D336" t="s">
         <v>7</v>
@@ -8643,10 +8655,10 @@
     </row>
     <row r="337" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="C337" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="D337" t="s">
         <v>7</v>
@@ -8654,10 +8666,10 @@
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="C338" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="D338" t="s">
         <v>7</v>
@@ -8665,10 +8677,10 @@
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>878</v>
+        <v>973</v>
       </c>
       <c r="C339" t="s">
-        <v>879</v>
+        <v>974</v>
       </c>
       <c r="D339" t="s">
         <v>7</v>
@@ -8676,10 +8688,10 @@
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>972</v>
+        <v>881</v>
       </c>
       <c r="C340" t="s">
-        <v>973</v>
+        <v>882</v>
       </c>
       <c r="D340" t="s">
         <v>7</v>
@@ -8687,10 +8699,10 @@
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>880</v>
+        <v>975</v>
       </c>
       <c r="C341" t="s">
-        <v>881</v>
+        <v>976</v>
       </c>
       <c r="D341" t="s">
         <v>7</v>
@@ -8698,10 +8710,10 @@
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="C342" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="D342" t="s">
         <v>7</v>
@@ -8709,13 +8721,10 @@
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>974</v>
-      </c>
-      <c r="B343" t="s">
-        <v>975</v>
+        <v>885</v>
       </c>
       <c r="C343" t="s">
-        <v>976</v>
+        <v>886</v>
       </c>
       <c r="D343" t="s">
         <v>7</v>
@@ -9045,13 +9054,13 @@
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>111</v>
+        <v>1046</v>
       </c>
       <c r="B367" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="C367" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="D367" t="s">
         <v>7</v>
@@ -9059,7 +9068,7 @@
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>1048</v>
+        <v>111</v>
       </c>
       <c r="B368" t="s">
         <v>1049</v>
@@ -9591,13 +9600,13 @@
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>237</v>
+        <v>1162</v>
       </c>
       <c r="B406" t="s">
-        <v>238</v>
+        <v>1163</v>
       </c>
       <c r="C406" t="s">
-        <v>239</v>
+        <v>1164</v>
       </c>
       <c r="D406" t="s">
         <v>7</v>
@@ -9605,13 +9614,13 @@
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B407" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C407" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D407" t="s">
         <v>7</v>
@@ -9619,13 +9628,13 @@
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>1162</v>
+        <v>240</v>
       </c>
       <c r="B408" t="s">
-        <v>1163</v>
+        <v>241</v>
       </c>
       <c r="C408" t="s">
-        <v>1164</v>
+        <v>242</v>
       </c>
       <c r="D408" t="s">
         <v>7</v>
@@ -9731,13 +9740,13 @@
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>243</v>
+        <v>1186</v>
       </c>
       <c r="B416" t="s">
-        <v>244</v>
+        <v>1187</v>
       </c>
       <c r="C416" t="s">
-        <v>245</v>
+        <v>1188</v>
       </c>
       <c r="D416" t="s">
         <v>7</v>
@@ -9745,13 +9754,13 @@
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B417" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C417" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D417" t="s">
         <v>7</v>
@@ -9759,13 +9768,13 @@
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B418" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C418" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D418" t="s">
         <v>7</v>
@@ -9773,13 +9782,13 @@
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B419" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C419" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D419" t="s">
         <v>7</v>
@@ -9787,13 +9796,13 @@
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B420" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C420" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D420" t="s">
         <v>7</v>
@@ -9801,13 +9810,13 @@
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B421" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C421" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D421" t="s">
         <v>7</v>
@@ -9815,13 +9824,13 @@
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B422" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C422" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D422" t="s">
         <v>7</v>
@@ -9829,13 +9838,13 @@
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="B423" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C423" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D423" t="s">
         <v>7</v>
@@ -9843,13 +9852,13 @@
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B424" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C424" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D424" t="s">
         <v>7</v>
@@ -9857,13 +9866,13 @@
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B425" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C425" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D425" t="s">
         <v>7</v>
@@ -9871,13 +9880,13 @@
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B426" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C426" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D426" t="s">
         <v>7</v>
@@ -9885,13 +9894,13 @@
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B427" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C427" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D427" t="s">
         <v>7</v>
@@ -9899,13 +9908,13 @@
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B428" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C428" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D428" t="s">
         <v>7</v>
@@ -9913,13 +9922,13 @@
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B429" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C429" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D429" t="s">
         <v>7</v>
@@ -9927,13 +9936,13 @@
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B430" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C430" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D430" t="s">
         <v>7</v>
@@ -9941,15 +9950,29 @@
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
+        <v>285</v>
+      </c>
+      <c r="B431" t="s">
+        <v>286</v>
+      </c>
+      <c r="C431" t="s">
+        <v>287</v>
+      </c>
+      <c r="D431" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="432" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A432" t="s">
         <v>288</v>
       </c>
-      <c r="B431" t="s">
+      <c r="B432" t="s">
         <v>289</v>
       </c>
-      <c r="C431" t="s">
+      <c r="C432" t="s">
         <v>290</v>
       </c>
-      <c r="D431" t="s">
+      <c r="D432" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>